<commit_message>
chore: verify costs with AWS price lists, FX 96.12; add .gitignore and README; drop Excel lock file
- Tracker Cost sheet: EC2, EBS gp3, public IPv4, KMS, Secrets Manager verified
  against AWS Price List API (ap-south-1); snapshot estimate corrected to $0.50
- Exchange rate 96.12 (median of Trading Economics, Wise, Frankfurter, 2026-10-02)
- Issue I-3 closed
- .gitignore: secrets, Terraform state/vars, Office lock files, private memory

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/Weekend2.0_Tracker.xlsx
+++ b/tracking/Weekend2.0_Tracker.xlsx
@@ -32,13 +32,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="7">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
-    <numFmt numFmtId="166" formatCode="₹#,##0;(₹#,##0);&quot;-&quot;"/>
-    <numFmt numFmtId="167" formatCode="$#,##0.00"/>
-    <numFmt numFmtId="168" formatCode="₹#,##0"/>
-    <numFmt numFmtId="169" formatCode="0.0%"/>
+    <numFmt numFmtId="165" formatCode="₹#,##0;(₹#,##0);&quot;-&quot;"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="$#,##0.00;($#,##0.00);&quot;-&quot;"/>
+    <numFmt numFmtId="168" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="169" formatCode="₹#,##0"/>
+    <numFmt numFmtId="170" formatCode="$#,##0.000;($#,##0.000);&quot;-&quot;"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -122,7 +123,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -136,8 +137,8 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -156,17 +157,31 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="168" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1185,7 +1200,7 @@
           <t>Estimated cost (₹)</t>
         </is>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="24">
         <f>Cost!D13</f>
         <v/>
       </c>
@@ -1198,7 +1213,7 @@
           <t>Budget (₹)</t>
         </is>
       </c>
-      <c r="B39" s="9">
+      <c r="B39" s="24">
         <f>Cost!B16</f>
         <v/>
       </c>
@@ -1211,7 +1226,7 @@
           <t>Headroom (₹)</t>
         </is>
       </c>
-      <c r="B40" s="9">
+      <c r="B40" s="24">
         <f>Cost!B17</f>
         <v/>
       </c>
@@ -1224,7 +1239,7 @@
           <t>Budget used</t>
         </is>
       </c>
-      <c r="B41" s="10">
+      <c r="B41" s="25">
         <f>Cost!B18</f>
         <v/>
       </c>
@@ -2599,18 +2614,20 @@
       </c>
       <c r="D4" s="13" t="inlineStr">
         <is>
-          <t>Refresh with the AWS Pricing Calculator before D1</t>
+          <t>Done 2026-10-02: EC2, EBS, IPv4, KMS, Secrets verified via AWS Price List API. S3/CloudWatch volumes remain estimates.</t>
         </is>
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F4" s="16" t="n">
         <v>46297</v>
       </c>
-      <c r="G4" s="14" t="n"/>
+      <c r="G4" s="14" t="n">
+        <v>46297</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -2795,19 +2812,23 @@
           <t>$0.0224/h × 730 h</t>
         </is>
       </c>
-      <c r="C2" s="17" t="n">
-        <v>16.35</v>
-      </c>
-      <c r="D2" s="18">
+      <c r="C2" s="26" t="n">
+        <v>16.352</v>
+      </c>
+      <c r="D2" s="27">
         <f>C2*$B$15</f>
         <v/>
       </c>
       <c r="E2" s="13" t="inlineStr">
         <is>
-          <t>sparecores.com (2026-10-02)</t>
-        </is>
-      </c>
-      <c r="F2" s="12" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>AWS Price List API, ap-south-1 (AmazonEC2, published 2026-09-25)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -2817,22 +2838,26 @@
       </c>
       <c r="B3" s="12" t="inlineStr">
         <is>
-          <t>~$0.09/GB-month</t>
-        </is>
-      </c>
-      <c r="C3" s="17" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="D3" s="18">
+          <t>$0.0912/GB-month × 40 GB</t>
+        </is>
+      </c>
+      <c r="C3" s="26" t="n">
+        <v>3.648</v>
+      </c>
+      <c r="D3" s="27">
         <f>C3*$B$15</f>
         <v/>
       </c>
       <c r="E3" s="13" t="inlineStr">
         <is>
-          <t>Estimate — check AWS Pricing Calculator</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>AWS Price List API, ap-south-1 (AmazonEC2/EBS, published 2026-09-25)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -2842,22 +2867,26 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>$0.005/h × 730 h</t>
-        </is>
-      </c>
-      <c r="C4" s="17" t="n">
+          <t>$0.005/h × 730 h (in-use IPv4)</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="n">
         <v>3.65</v>
       </c>
-      <c r="D4" s="18">
+      <c r="D4" s="27">
         <f>C4*$B$15</f>
         <v/>
       </c>
       <c r="E4" s="13" t="inlineStr">
         <is>
-          <t>Estimate — check AWS Pricing Calculator</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>AWS Price List API, ap-south-1 (AmazonVPC, published 2026-09-17)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -2867,22 +2896,26 @@
       </c>
       <c r="B5" s="12" t="inlineStr">
         <is>
-          <t>2 keys × $1</t>
-        </is>
-      </c>
-      <c r="C5" s="17" t="n">
+          <t>2 keys × $1/month (+$0.03 per 10k requests)</t>
+        </is>
+      </c>
+      <c r="C5" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="27">
         <f>C5*$B$15</f>
         <v/>
       </c>
       <c r="E5" s="13" t="inlineStr">
         <is>
-          <t>Estimate — check AWS Pricing Calculator</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>AWS Price List API, ap-south-1 (awskms, published 2026-09-11)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -2892,22 +2925,26 @@
       </c>
       <c r="B6" s="12" t="inlineStr">
         <is>
-          <t>5 secrets × $0.40</t>
-        </is>
-      </c>
-      <c r="C6" s="17" t="n">
+          <t>5 secrets × $0.40 (+$0.05 per 10k API calls)</t>
+        </is>
+      </c>
+      <c r="C6" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="27">
         <f>C6*$B$15</f>
         <v/>
       </c>
       <c r="E6" s="13" t="inlineStr">
         <is>
-          <t>Estimate — check AWS Pricing Calculator</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="n"/>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>AWS Price List API, ap-south-1 (AWSSecretsManager, published 2026-09-11)</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -2917,22 +2954,26 @@
       </c>
       <c r="B7" s="12" t="inlineStr">
         <is>
-          <t>~15 GB + requests</t>
-        </is>
-      </c>
-      <c r="C7" s="17" t="n">
+          <t>~15 GB × $0.025/GB-month + requests</t>
+        </is>
+      </c>
+      <c r="C7" s="26" t="n">
         <v>0.6</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="27">
         <f>C7*$B$15</f>
         <v/>
       </c>
       <c r="E7" s="13" t="inlineStr">
         <is>
-          <t>DESIGN.md §21.2</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="n"/>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>Rate: AWS Price List API, ap-south-1 (AmazonS3 Standard first 50 TB); volume estimated</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -2942,22 +2983,26 @@
       </c>
       <c r="B8" s="12" t="inlineStr">
         <is>
-          <t>Weekly, incremental</t>
-        </is>
-      </c>
-      <c r="C8" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="18">
+          <t>$0.05/GB-month × ~10 GB</t>
+        </is>
+      </c>
+      <c r="C8" s="26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D8" s="27">
         <f>C8*$B$15</f>
         <v/>
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>DESIGN.md §21.2</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="n"/>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>Rate: AWS Price List API, ap-south-1 (EBS snapshots, 2026-09-25); size estimated</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -2967,22 +3012,26 @@
       </c>
       <c r="B9" s="12" t="inlineStr">
         <is>
-          <t>&lt; 1 GB/month</t>
-        </is>
-      </c>
-      <c r="C9" s="17" t="n">
+          <t>&lt; 1 GB: $0.67/GB ingest + $0.03/GB-month</t>
+        </is>
+      </c>
+      <c r="C9" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="27">
         <f>C9*$B$15</f>
         <v/>
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>DESIGN.md §21.2</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="n"/>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>Rate: AWS Price List API, ap-south-1 (AmazonCloudWatch); volume estimated</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -2995,10 +3044,10 @@
           <t>Personal plan</t>
         </is>
       </c>
-      <c r="C10" s="17" t="n">
+      <c r="C10" s="28" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="27">
         <f>C10*$B$15</f>
         <v/>
       </c>
@@ -3020,10 +3069,10 @@
           <t>80% Haiku 4.5 / 20% Sonnet 5, +10% regional</t>
         </is>
       </c>
-      <c r="C11" s="17" t="n">
+      <c r="C11" s="28" t="n">
         <v>15.9</v>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="27">
         <f>C11*$B$15</f>
         <v/>
       </c>
@@ -3041,11 +3090,11 @@
         </is>
       </c>
       <c r="B13" s="5" t="n"/>
-      <c r="C13" s="19">
+      <c r="C13" s="29">
         <f>SUM(C2:C11)</f>
         <v/>
       </c>
-      <c r="D13" s="20">
+      <c r="D13" s="30">
         <f>SUM(D2:D11)</f>
         <v/>
       </c>
@@ -3063,11 +3112,11 @@
         </is>
       </c>
       <c r="B15" s="21" t="n">
-        <v>96.3</v>
+        <v>96.12</v>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>Mid-market, 2026-10-02, tradingeconomics.com</t>
+          <t>Median mid-market, 2026-10-02 ~20:10 IST: Trading Economics 96.1210 · Wise 96.0682 · Frankfurter 96.14. FBIL reference not published (Gandhi Jayanti holiday).</t>
         </is>
       </c>
       <c r="D15" s="5" t="n"/>
@@ -3078,7 +3127,7 @@
           <t>Monthly budget (₹)</t>
         </is>
       </c>
-      <c r="B16" s="22" t="n">
+      <c r="B16" s="31" t="n">
         <v>5000</v>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -3094,7 +3143,7 @@
           <t>Headroom (₹)</t>
         </is>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="24">
         <f>B16-D13</f>
         <v/>
       </c>
@@ -3107,7 +3156,7 @@
           <t>Budget used</t>
         </is>
       </c>
-      <c r="B18" s="10">
+      <c r="B18" s="25">
         <f>IFERROR(D13/B16,0)</f>
         <v/>
       </c>
@@ -3246,7 +3295,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3383,6 +3432,31 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Costs verified against AWS Price List API (ap-south-1); FX 96.12; I-3 closed</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:E5"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(infra): draft Terraform for D1 option E2 (revised); tracker Resources + Automation Scripts sheets
- infra/: bootstrap state bucket + 9 modules (network, kms, secrets, database,
  app, scheduler, entry_node, backup, budget) and envs/prod
- Validated with Terraform 1.16.5 and AWS provider 6.67.0; lock files for
  darwin_arm64 + linux_amd64
- Serverless-first: Lambda (python3.14, arm64) behind an AWS_IAM Function URL,
  Aurora Serverless v2 (scale to zero, Data API), Bedrock India profiles,
  EventBridge Scheduler (IST), t4g.nano tailnet entry node with no inbound ports
- Tracker: Resources sheet (39 lines, ~USD 42.80 / INR 4,114 per month),
  Automation Scripts sheet (21 Python scripts), tasks T-016..T-019, issues I-7, I-8

PROVISIONAL: depends on decision D1. Not applied.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/Weekend2.0_Tracker.xlsx
+++ b/tracking/Weekend2.0_Tracker.xlsx
@@ -14,8 +14,10 @@
     <sheet name="Decisions" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Issues" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Cost" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Approvals" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Doc versions" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Resources" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Automation Scripts" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Approvals" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Doc versions" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Phases'!$A$1:$J$8</definedName>
@@ -23,8 +25,10 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Decisions'!$A$1:$H$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Issues'!$A$1:$G$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cost'!$A$1:$F$11</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Approvals'!$A$1:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Doc versions'!$A$1:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Resources'!$A$1:$N$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Automation Scripts'!$A$1:$L$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Approvals'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Doc versions'!$A$1:$E$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -123,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -182,6 +186,9 @@
     <xf numFmtId="168" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="169" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -736,13 +743,291 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Action</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Approved by</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>Send architecture design (no secrets/personal data) to Figma</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>Figma Inc. (FigJam)</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E2"/>
+  <dataValidations count="1">
+    <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Low,Medium,High"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="70" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Document</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Version</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="13" t="inlineStr">
+        <is>
+          <t>DESIGN.md</t>
+        </is>
+      </c>
+      <c r="B2" s="13" t="inlineStr">
+        <is>
+          <t>0.1.0</t>
+        </is>
+      </c>
+      <c r="C2" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>Initial draft</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>Base plan: architecture, components, cost model, roadmap</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>DESIGN.md</t>
+        </is>
+      </c>
+      <c r="B3" s="13" t="inlineStr">
+        <is>
+          <t>0.1.1</t>
+        </is>
+      </c>
+      <c r="C3" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D3" s="13" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>Budget set to ₹5,000/month; budget fit added</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>DESIGN.md</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>0.1.2</t>
+        </is>
+      </c>
+      <c r="C4" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="E4" s="13" t="inlineStr">
+        <is>
+          <t>FigJam board link; data exit X8 (Figma)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>DESIGN.md</t>
+        </is>
+      </c>
+      <c r="B5" s="13" t="inlineStr">
+        <is>
+          <t>0.1.3</t>
+        </is>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="E5" s="13" t="inlineStr">
+        <is>
+          <t>Diagram images added (docs/diagrams/: jpg, svg, mmd)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C6" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D6" s="13" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="E6" s="13" t="inlineStr">
+        <is>
+          <t>Costs verified against AWS Price List API (ap-south-1); FX 96.12; I-3 closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B7" s="13" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="C7" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D7" s="13" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E7" s="13" t="inlineStr">
+        <is>
+          <t>Resources sheet (39 lines, E2 Terraform) + Automation Scripts sheet (21 scripts); tasks T-016–T-019; issues I-7, I-8</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E5"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:D50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1258,6 +1543,79 @@
       </c>
       <c r="C42" s="5" t="n"/>
       <c r="D42" s="5" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>Infrastructure (Terraform — PROVISIONAL)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>Resources tracked</t>
+        </is>
+      </c>
+      <c r="B45" s="5">
+        <f>COUNTA(Resources!$B$2:$B$40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>Resources applied</t>
+        </is>
+      </c>
+      <c r="B46" s="5">
+        <f>COUNTIF(Resources!$M$2:$M$200,"Applied")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>E2 estimated cost (₹/month)</t>
+        </is>
+      </c>
+      <c r="B47" s="32">
+        <f>Resources!J42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>E2 fits budget?</t>
+        </is>
+      </c>
+      <c r="B48" s="5">
+        <f>Resources!J45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>Automation scripts planned</t>
+        </is>
+      </c>
+      <c r="B49" s="5">
+        <f>COUNTA('Automation Scripts'!$A$2:$A$22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>High-priority scripts not done</t>
+        </is>
+      </c>
+      <c r="B50" s="5">
+        <f>COUNTIFS('Automation Scripts'!$J$2:$J$200,"High",'Automation Scripts'!$K$2:$K$200,"&lt;&gt;Done")</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B2:B200">
@@ -1292,6 +1650,14 @@
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B48">
+    <cfRule type="cellIs" priority="9" operator="equal" dxfId="0">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="10" operator="equal" dxfId="2">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -1631,7 +1997,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2005,7 +2371,11 @@
       <c r="F10" s="14" t="n"/>
       <c r="G10" s="14" t="n"/>
       <c r="H10" s="14" t="n"/>
-      <c r="I10" s="13" t="inlineStr"/>
+      <c r="I10" s="13" t="inlineStr">
+        <is>
+          <t>E2 (revised) recommended; Terraform drafted for it</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -2194,6 +2564,138 @@
       <c r="G16" s="14" t="n"/>
       <c r="H16" s="14" t="n"/>
       <c r="I16" s="13" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>T-016</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Draft Terraform (E2 revised): 9 modules + bootstrap; validated (TF 1.16.5, AWS 6.67.0)</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F17" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G17" s="14" t="n"/>
+      <c r="H17" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>infra/ — PROVISIONAL until D1</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>T-017</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Plan Python automation scripts (21) — Automation Scripts sheet</t>
+        </is>
+      </c>
+      <c r="D18" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E18" s="13" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G18" s="14" t="n"/>
+      <c r="H18" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="I18" s="13" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>T-018</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Confirm Aurora engine version + Bedrock India model IDs in ap-south-1</t>
+        </is>
+      </c>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F19" s="14" t="n"/>
+      <c r="G19" s="14" t="n"/>
+      <c r="H19" s="14" t="n"/>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>Commands in infra/README.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>T-019</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Upgrade local Terraform 1.5.7 → 1.16.x (hashicorp/tap)</t>
+        </is>
+      </c>
+      <c r="D20" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F20" s="14" t="n"/>
+      <c r="G20" s="14" t="n"/>
+      <c r="H20" s="14" t="n"/>
+      <c r="I20" s="13" t="inlineStr"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:I16"/>
@@ -2485,7 +2987,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2721,6 +3223,68 @@
         <v>46297</v>
       </c>
       <c r="G7" s="14" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>I-7</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Aurora resumes in ~15 s (30 s+ after 24 h idle) — first message after a pause is slow</t>
+        </is>
+      </c>
+      <c r="C8" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Accept, or raise min ACU (cost) — decide with D5</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F8" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G8" s="14" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>I-8</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Exact Bedrock India profile ID for Sonnet 5 not verified</t>
+        </is>
+      </c>
+      <c r="C9" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>Run list-inference-profiles (T-018)</t>
+        </is>
+      </c>
+      <c r="E9" s="13" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G9" s="14" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G7"/>
@@ -2758,7 +3322,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -3180,6 +3744,13 @@
       <c r="A21" s="23" t="inlineStr">
         <is>
           <t>Scope: text-only, Option B (private EC2 + Bedrock). Voice adds ≈ ₹1,580 (local) or ≈ ₹3,040 (AWS) — see DESIGN.md §21.3–21.4.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
+        <is>
+          <t>Note: this sheet is the option-B baseline. The E2 (revised) Terraform estimate is on the Resources sheet; switch after D1.</t>
         </is>
       </c>
     </row>
@@ -3216,73 +3787,2722 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:N47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="60" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="40" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="48" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B1" s="11" t="inlineStr">
         <is>
-          <t>Action</t>
+          <t>Terraform address</t>
         </is>
       </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>Target</t>
+          <t>AWS resource</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
         <is>
-          <t>Risk</t>
+          <t>Name</t>
         </is>
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Approved by</t>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>Region / AZ</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Key settings</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>USD / month</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>INR / month</t>
+        </is>
+      </c>
+      <c r="K1" s="11" t="inlineStr">
+        <is>
+          <t>Price basis / source</t>
+        </is>
+      </c>
+      <c r="L1" s="11" t="inlineStr">
+        <is>
+          <t>Verified?</t>
+        </is>
+      </c>
+      <c r="M1" s="11" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="N1" s="11" t="inlineStr">
+        <is>
+          <t>Phase</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="n">
-        <v>46297</v>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>Send architecture design (no secrets/personal data) to Figma</t>
-        </is>
-      </c>
-      <c r="C2" s="13" t="inlineStr">
-        <is>
-          <t>Figma Inc. (FigJam)</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>Owner</t>
+      <c r="A2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>module.network.aws_vpc.this</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>VPC</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-vpc</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>Private network</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>10.20.0.0/16; DNS hostnames on</t>
+        </is>
+      </c>
+      <c r="I2" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="27">
+        <f>I2*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K2" s="12" t="inlineStr">
+        <is>
+          <t>No charge for VPCs</t>
+        </is>
+      </c>
+      <c r="L2" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M2" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N2" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>module.network.aws_default_security_group.this</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Security group</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-default-sg-locked</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>Lock the default SG</t>
+        </is>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>No rules at all</t>
+        </is>
+      </c>
+      <c r="I3" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" s="27">
+        <f>I3*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K3" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L3" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M3" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N3" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>module.network.aws_internet_gateway.this</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Internet gateway</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-igw</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>Egress for the entry node</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I4" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" s="27">
+        <f>I4*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K4" s="12" t="inlineStr">
+        <is>
+          <t>No charge (data transfer separate)</t>
+        </is>
+      </c>
+      <c r="L4" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M4" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N4" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>module.network.aws_subnet.public_a</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Subnet</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-public-a</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1a</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>Entry node only</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>10.20.0.0/24; no auto public IP</t>
+        </is>
+      </c>
+      <c r="I5" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="27">
+        <f>I5*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K5" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>module.network.aws_subnet.private["a"]</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Subnet</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-private-a</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1a</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>Aurora</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>10.20.10.0/24; no internet route</t>
+        </is>
+      </c>
+      <c r="I6" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="27">
+        <f>I6*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K6" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L6" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M6" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N6" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>module.network.aws_subnet.private["b"]</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Subnet</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-private-b</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1b</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>Aurora (2nd AZ required)</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>10.20.11.0/24; no internet route</t>
+        </is>
+      </c>
+      <c r="I7" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" s="27">
+        <f>I7*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K7" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L7" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M7" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N7" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>module.network.aws_route_table.public</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Route table</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-public-rt</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>Public routing</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>0.0.0.0/0 → IGW</t>
+        </is>
+      </c>
+      <c r="I8" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="27">
+        <f>I8*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L8" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M8" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N8" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>module.network.aws_route_table.private</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Route table</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-private-rt</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>network</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>Private routing</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>Local routes only; no NAT</t>
+        </is>
+      </c>
+      <c r="I9" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" s="27">
+        <f>I9*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L9" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M9" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>module.kms.aws_kms_key.data</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>KMS key (CMK)</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-data</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>kms</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>Encrypts Aurora, secrets, logs, EBS, S3 (P3)</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>Rotation 365 d; 30 d deletion window</t>
+        </is>
+      </c>
+      <c r="I10" s="26" t="n">
+        <v>1</v>
+      </c>
+      <c r="J10" s="27">
+        <f>I10*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K10" s="12" t="inlineStr">
+        <is>
+          <t>$1/key-month (AWS Price List API ap-south-1 2026-09-11)</t>
+        </is>
+      </c>
+      <c r="L10" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M10" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>module.kms.aws_kms_alias.data</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>KMS alias</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>alias/weekend2-prod-data</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>kms</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>Friendly key name</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I11" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" s="27">
+        <f>I11*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K11" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L11" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M11" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>module.secrets.aws_secretsmanager_secret.this["tailscale/authkey"]</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod/tailscale/authkey</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>secrets</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>Entry node joins tailnet (P4)</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>KMS; 7-day recovery</t>
+        </is>
+      </c>
+      <c r="I12" s="26" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J12" s="27">
+        <f>I12*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K12" s="12" t="inlineStr">
+        <is>
+          <t>$0.40/secret-month (AWS Price List API ap-south-1 2026-09-11)</t>
+        </is>
+      </c>
+      <c r="L12" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M12" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>module.secrets.aws_secretsmanager_secret.this["app/session-signing-key"]</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod/app/session-signing-key</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>secrets</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>Passkey session cookies</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>KMS</t>
+        </is>
+      </c>
+      <c r="I13" s="26" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J13" s="27">
+        <f>I13*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K13" s="12" t="inlineStr">
+        <is>
+          <t>$0.40/secret-month</t>
+        </is>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M13" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N13" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>module.secrets.aws_secretsmanager_secret.this["connectors/google-oauth-client"]</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod/connectors/google-oauth-client</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>secrets</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>Calendar/Gmail connectors</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>KMS; value set in Phase 3</t>
+        </is>
+      </c>
+      <c r="I14" s="26" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J14" s="27">
+        <f>I14*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K14" s="12" t="inlineStr">
+        <is>
+          <t>$0.40/secret-month</t>
+        </is>
+      </c>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M14" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N14" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>(RDS-managed, via aws_rds_cluster)</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>rds!cluster-&lt;id&gt; (auto-named)</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>Aurora master password, rotated by RDS</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>KMS CMK</t>
+        </is>
+      </c>
+      <c r="I15" s="26" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J15" s="27">
+        <f>I15*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K15" s="12" t="inlineStr">
+        <is>
+          <t>$0.40/secret-month</t>
+        </is>
+      </c>
+      <c r="L15" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M15" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>module.database.aws_db_subnet_group.this</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>DB subnet group</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-aurora-subnets</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1a/1b</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>Aurora placement</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>private-a + private-b</t>
+        </is>
+      </c>
+      <c r="I16" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="27">
+        <f>I16*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K16" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L16" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M16" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>module.database.aws_security_group.aurora</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Security group</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-aurora-sg</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>No network access</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>No ingress; Data API only</t>
+        </is>
+      </c>
+      <c r="I17" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" s="27">
+        <f>I17*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K17" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M17" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N17" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>module.database.aws_rds_cluster.this</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Aurora PostgreSQL Serverless v2</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-aurora</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1a/1b</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>Conversations, memories (pgvector)</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>0–2 ACU; auto-pause 300 s; Data API; KMS; deletion protection; 7-day backups</t>
+        </is>
+      </c>
+      <c r="I18" s="26" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="J18" s="27">
+        <f>I18*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K18" s="12" t="inlineStr">
+        <is>
+          <t>$0.18/ACU-h (AWS Price List API ap-south-1) × 0.5 ACU × ~6 h/day × 30 — hours ESTIMATED</t>
+        </is>
+      </c>
+      <c r="L18" s="13" t="inlineStr">
+        <is>
+          <t>Rate verified; usage estimate</t>
+        </is>
+      </c>
+      <c r="M18" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N18" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>module.database.aws_rds_cluster_instance.writer</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>DB instance</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-aurora-1</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>Writer</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>db.serverless; not public</t>
+        </is>
+      </c>
+      <c r="I19" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="27">
+        <f>I19*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K19" s="12" t="inlineStr">
+        <is>
+          <t>Billed as cluster ACU</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M19" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N19" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>(Aurora storage + I/O)</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Data at rest</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>Encrypted</t>
+        </is>
+      </c>
+      <c r="I20" s="26" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="J20" s="27">
+        <f>I20*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K20" s="12" t="inlineStr">
+        <is>
+          <t>~2 GB × $0.11/GB-mo + ~1M I/O × $0.22/M (rates verified)</t>
+        </is>
+      </c>
+      <c r="L20" s="13" t="inlineStr">
+        <is>
+          <t>Rate verified; volume estimate</t>
+        </is>
+      </c>
+      <c r="M20" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N20" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>module.app.aws_lambda_function.api</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Lambda</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-api</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>Chat, voice, memory API</t>
+        </is>
+      </c>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>python3.14; arm64; 1024 MB; 60 s; KMS env</t>
+        </is>
+      </c>
+      <c r="I21" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" s="27">
+        <f>I21*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K21" s="12" t="inlineStr">
+        <is>
+          <t>Within free tier (1M req + 400k GB-s/mo); beyond: $0.0000133334/GB-s ARM (verified)</t>
+        </is>
+      </c>
+      <c r="L21" s="13" t="inlineStr">
+        <is>
+          <t>Rate verified; free tier Not verified</t>
+        </is>
+      </c>
+      <c r="M21" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N21" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>module.app.aws_lambda_function_url.api</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Lambda Function URL</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-api (URL)</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>Private entry for the API</t>
+        </is>
+      </c>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>AWS_IAM auth; RESPONSE_STREAM</t>
+        </is>
+      </c>
+      <c r="I22" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" s="27">
+        <f>I22*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K22" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L22" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M22" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N22" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>module.app.aws_iam_role.api</t>
+        </is>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>IAM role</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-api-role</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="F23" s="12" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="G23" s="12" t="inlineStr">
+        <is>
+          <t>API permissions</t>
+        </is>
+      </c>
+      <c r="H23" s="12" t="inlineStr">
+        <is>
+          <t>Data API, own secrets, KMS, Bedrock in.*, reminder schedules</t>
+        </is>
+      </c>
+      <c r="I23" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="27">
+        <f>I23*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K23" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L23" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M23" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N23" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>module.app.aws_cloudwatch_log_group.api</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>Log group</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>/aws/lambda/weekend2-prod-api</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="F24" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G24" s="12" t="inlineStr">
+        <is>
+          <t>API logs (no message content)</t>
+        </is>
+      </c>
+      <c r="H24" s="12" t="inlineStr">
+        <is>
+          <t>14 days; KMS; JSON</t>
+        </is>
+      </c>
+      <c r="I24" s="26" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="J24" s="27">
+        <f>I24*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K24" s="12" t="inlineStr">
+        <is>
+          <t>$0.67/GB ingest + $0.03/GB-mo (verified); volume estimate</t>
+        </is>
+      </c>
+      <c r="L24" s="13" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="M24" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N24" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>module.app.aws_lambda_function.worker</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Lambda</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-worker</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="F25" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G25" s="12" t="inlineStr">
+        <is>
+          <t>Scheduled jobs</t>
+        </is>
+      </c>
+      <c r="H25" s="12" t="inlineStr">
+        <is>
+          <t>python3.14; arm64; 512 MB; 300 s</t>
+        </is>
+      </c>
+      <c r="I25" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" s="27">
+        <f>I25*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K25" s="12" t="inlineStr">
+        <is>
+          <t>Within free tier</t>
+        </is>
+      </c>
+      <c r="L25" s="13" t="inlineStr">
+        <is>
+          <t>Rate verified; free tier Not verified</t>
+        </is>
+      </c>
+      <c r="M25" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N25" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>module.app.aws_iam_role.worker</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>IAM role</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-worker-role</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="F26" s="12" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="G26" s="12" t="inlineStr">
+        <is>
+          <t>Worker permissions</t>
+        </is>
+      </c>
+      <c r="H26" s="12" t="inlineStr">
+        <is>
+          <t>Data API, secrets, KMS, backup bucket</t>
+        </is>
+      </c>
+      <c r="I26" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="27">
+        <f>I26*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K26" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L26" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M26" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N26" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="12" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="12" t="inlineStr">
+        <is>
+          <t>module.app.aws_cloudwatch_log_group.worker</t>
+        </is>
+      </c>
+      <c r="C27" s="12" t="inlineStr">
+        <is>
+          <t>Log group</t>
+        </is>
+      </c>
+      <c r="D27" s="12" t="inlineStr">
+        <is>
+          <t>/aws/lambda/weekend2-prod-worker</t>
+        </is>
+      </c>
+      <c r="E27" s="12" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="F27" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G27" s="12" t="inlineStr">
+        <is>
+          <t>Worker logs</t>
+        </is>
+      </c>
+      <c r="H27" s="12" t="inlineStr">
+        <is>
+          <t>14 days; KMS</t>
+        </is>
+      </c>
+      <c r="I27" s="26" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="J27" s="27">
+        <f>I27*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K27" s="12" t="inlineStr">
+        <is>
+          <t>$0.67/GB ingest; volume estimate</t>
+        </is>
+      </c>
+      <c r="L27" s="13" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="M27" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N27" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>module.scheduler.aws_scheduler_schedule_group.this</t>
+        </is>
+      </c>
+      <c r="C28" s="12" t="inlineStr">
+        <is>
+          <t>Schedule group</t>
+        </is>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod</t>
+        </is>
+      </c>
+      <c r="E28" s="12" t="inlineStr">
+        <is>
+          <t>scheduler</t>
+        </is>
+      </c>
+      <c r="F28" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G28" s="12" t="inlineStr">
+        <is>
+          <t>Holds daily + reminder schedules</t>
+        </is>
+      </c>
+      <c r="H28" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I28" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="27">
+        <f>I28*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K28" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L28" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M28" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N28" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>module.scheduler.aws_scheduler_schedule.daily["retention"]</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-retention-daily</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>scheduler</t>
+        </is>
+      </c>
+      <c r="F29" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G29" s="12" t="inlineStr">
+        <is>
+          <t>Retention cleanup (P5)</t>
+        </is>
+      </c>
+      <c r="H29" s="12" t="inlineStr">
+        <is>
+          <t>cron 03:00 Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="I29" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J29" s="27">
+        <f>I29*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K29" s="12" t="inlineStr">
+        <is>
+          <t>Free tier 14M invocations/mo</t>
+        </is>
+      </c>
+      <c r="L29" s="13" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="M29" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N29" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>module.scheduler.aws_scheduler_schedule.daily["export"]</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Schedule</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-export-daily</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>scheduler</t>
+        </is>
+      </c>
+      <c r="F30" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G30" s="12" t="inlineStr">
+        <is>
+          <t>Encrypted export (P6/P10)</t>
+        </is>
+      </c>
+      <c r="H30" s="12" t="inlineStr">
+        <is>
+          <t>cron 03:30 Asia/Kolkata</t>
+        </is>
+      </c>
+      <c r="I30" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="27">
+        <f>I30*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K30" s="12" t="inlineStr">
+        <is>
+          <t>Free tier 14M invocations/mo</t>
+        </is>
+      </c>
+      <c r="L30" s="13" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="M30" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N30" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>module.scheduler.aws_iam_role.scheduler</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>IAM role</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-scheduler-role</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>scheduler</t>
+        </is>
+      </c>
+      <c r="F31" s="12" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="G31" s="12" t="inlineStr">
+        <is>
+          <t>Scheduler → worker</t>
+        </is>
+      </c>
+      <c r="H31" s="12" t="inlineStr">
+        <is>
+          <t>lambda:InvokeFunction on worker only</t>
+        </is>
+      </c>
+      <c r="I31" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="27">
+        <f>I31*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K31" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L31" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M31" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N31" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>module.entry_node.aws_instance.this</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>EC2 t4g.nano</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-entry (tailnet: node-a1)</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>entry_node</t>
+        </is>
+      </c>
+      <c r="F32" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1a</t>
+        </is>
+      </c>
+      <c r="G32" s="12" t="inlineStr">
+        <is>
+          <t>Only server: tailnet entry + SigV4 forwarder</t>
+        </is>
+      </c>
+      <c r="H32" s="12" t="inlineStr">
+        <is>
+          <t>AL2023 arm64; IMDSv2; no inbound; SSM; standard credits</t>
+        </is>
+      </c>
+      <c r="I32" s="26" t="n">
+        <v>2.044</v>
+      </c>
+      <c r="J32" s="27">
+        <f>I32*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K32" s="12" t="inlineStr">
+        <is>
+          <t>$0.0028/h × 730 (AWS Price List API ap-south-1 2026-09-25)</t>
+        </is>
+      </c>
+      <c r="L32" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M32" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N32" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>(root_block_device of aws_instance.this)</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>EBS gp3 8 GB</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>entry_node</t>
+        </is>
+      </c>
+      <c r="F33" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1a</t>
+        </is>
+      </c>
+      <c r="G33" s="12" t="inlineStr">
+        <is>
+          <t>Root disk</t>
+        </is>
+      </c>
+      <c r="H33" s="12" t="inlineStr">
+        <is>
+          <t>Encrypted with CMK</t>
+        </is>
+      </c>
+      <c r="I33" s="26" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="J33" s="27">
+        <f>I33*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K33" s="12" t="inlineStr">
+        <is>
+          <t>$0.0912/GB-mo × 8 (2026-09-25)</t>
+        </is>
+      </c>
+      <c r="L33" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M33" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N33" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>(associate_public_ip_address)</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Public IPv4</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>entry_node</t>
+        </is>
+      </c>
+      <c r="F34" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1a</t>
+        </is>
+      </c>
+      <c r="G34" s="12" t="inlineStr">
+        <is>
+          <t>Egress only (no inbound rules)</t>
+        </is>
+      </c>
+      <c r="H34" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I34" s="26" t="n">
+        <v>3.65</v>
+      </c>
+      <c r="J34" s="27">
+        <f>I34*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K34" s="12" t="inlineStr">
+        <is>
+          <t>$0.005/h × 730 (AmazonVPC 2026-09-17)</t>
+        </is>
+      </c>
+      <c r="L34" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M34" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N34" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>module.entry_node.aws_security_group.entry</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Security group</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-entry-sg</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>entry_node</t>
+        </is>
+      </c>
+      <c r="F35" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G35" s="12" t="inlineStr">
+        <is>
+          <t>Egress-only firewall</t>
+        </is>
+      </c>
+      <c r="H35" s="12" t="inlineStr">
+        <is>
+          <t>Out: 443/tcp, 41641/udp, 3478/udp</t>
+        </is>
+      </c>
+      <c r="I35" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="27">
+        <f>I35*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K35" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L35" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M35" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N35" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>module.entry_node.aws_iam_role.entry + instance profile</t>
+        </is>
+      </c>
+      <c r="C36" s="12" t="inlineStr">
+        <is>
+          <t>IAM role/profile</t>
+        </is>
+      </c>
+      <c r="D36" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-entry-role / weekend2-prod-entry-profile</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>entry_node</t>
+        </is>
+      </c>
+      <c r="F36" s="12" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="G36" s="12" t="inlineStr">
+        <is>
+          <t>SSM + read Tailscale key + call API URL</t>
+        </is>
+      </c>
+      <c r="H36" s="12" t="inlineStr">
+        <is>
+          <t>Least privilege</t>
+        </is>
+      </c>
+      <c r="I36" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="27">
+        <f>I36*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K36" s="12" t="inlineStr">
+        <is>
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="L36" s="13" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="M36" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N36" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>module.backup.aws_s3_bucket.this</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>S3 bucket</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-backups-&lt;account-id&gt;</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>backup</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="inlineStr">
+        <is>
+          <t>Exports, audit copies, restore drills</t>
+        </is>
+      </c>
+      <c r="H37" s="12" t="inlineStr">
+        <is>
+          <t>Object Lock governance 35 d; SSE-KMS; versioning; TLS-only; lifecycle</t>
+        </is>
+      </c>
+      <c r="I37" s="26" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="J37" s="27">
+        <f>I37*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K37" s="12" t="inlineStr">
+        <is>
+          <t>~15 GB × $0.025/GB-mo (verified) + requests</t>
+        </is>
+      </c>
+      <c r="L37" s="13" t="inlineStr">
+        <is>
+          <t>Rate verified; volume estimate</t>
+        </is>
+      </c>
+      <c r="M37" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N37" s="12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="12" t="inlineStr">
+        <is>
+          <t>module.budget.aws_budgets_budget.monthly</t>
+        </is>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>AWS Budget</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-prod-monthly</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>budget</t>
+        </is>
+      </c>
+      <c r="F38" s="12" t="inlineStr">
+        <is>
+          <t>global</t>
+        </is>
+      </c>
+      <c r="G38" s="12" t="inlineStr">
+        <is>
+          <t>Cost alerts</t>
+        </is>
+      </c>
+      <c r="H38" s="12" t="inlineStr">
+        <is>
+          <t>USD 52; alerts 50/80/100% + forecast</t>
+        </is>
+      </c>
+      <c r="I38" s="26" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="27">
+        <f>I38*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K38" s="12" t="inlineStr">
+        <is>
+          <t>First 2 budgets free</t>
+        </is>
+      </c>
+      <c r="L38" s="13" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="M38" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N38" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="12" t="inlineStr">
+        <is>
+          <t>bootstrap: aws_s3_bucket.tfstate</t>
+        </is>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>S3 bucket</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-tfstate-&lt;account-id&gt;</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>bootstrap</t>
+        </is>
+      </c>
+      <c r="F39" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1</t>
+        </is>
+      </c>
+      <c r="G39" s="12" t="inlineStr">
+        <is>
+          <t>Terraform state + native lock</t>
+        </is>
+      </c>
+      <c r="H39" s="12" t="inlineStr">
+        <is>
+          <t>Versioning; SSE-KMS; TLS-only; prevent_destroy</t>
+        </is>
+      </c>
+      <c r="I39" s="26" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="J39" s="27">
+        <f>I39*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K39" s="12" t="inlineStr">
+        <is>
+          <t>KB-sized state</t>
+        </is>
+      </c>
+      <c r="L39" s="13" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="M39" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N39" s="12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="12" t="inlineStr">
+        <is>
+          <t>(no resource — IAM only)</t>
+        </is>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>Amazon Bedrock usage</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>Claude Haiku 4.5 / Sonnet 5 via in.* profiles</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="inlineStr">
+        <is>
+          <t>app</t>
+        </is>
+      </c>
+      <c r="F40" s="12" t="inlineStr">
+        <is>
+          <t>ap-south-1/2</t>
+        </is>
+      </c>
+      <c r="G40" s="12" t="inlineStr">
+        <is>
+          <t>LLM inference</t>
+        </is>
+      </c>
+      <c r="H40" s="12" t="inlineStr">
+        <is>
+          <t>India geo; +10% regional premium</t>
+        </is>
+      </c>
+      <c r="I40" s="26" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="J40" s="27">
+        <f>I40*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K40" s="12" t="inlineStr">
+        <is>
+          <t>DESIGN.md §21.1 (expected 3,000 turns)</t>
+        </is>
+      </c>
+      <c r="L40" s="13" t="inlineStr">
+        <is>
+          <t>Calculated (I-2 open)</t>
+        </is>
+      </c>
+      <c r="M40" s="13" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+      <c r="N40" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Total per month (expected use)</t>
+        </is>
+      </c>
+      <c r="I42" s="33">
+        <f>SUM(I2:I40)</f>
+        <v/>
+      </c>
+      <c r="J42" s="34">
+        <f>SUM(J2:J40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Budget (₹)</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="n"/>
+      <c r="J43" s="34">
+        <f>Cost!B16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Headroom (₹)</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="n"/>
+      <c r="J44" s="34">
+        <f>J43-J42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Fits budget?</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="n"/>
+      <c r="J45" s="3">
+        <f>IF(J42&lt;=J43,"Yes","No")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="23" t="inlineStr">
+        <is>
+          <t>Design: D1 option E2 (revised) — PROVISIONAL until D1 is decided. Source: infra/ (Terraform 1.16.5 / AWS provider 6.67.0, validated 2026-10-02). INR uses Cost!B15. Aurora hours are the main uncertainty.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E2"/>
+  <autoFilter ref="A1:N40"/>
+  <conditionalFormatting sqref="J45">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Yes"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="2">
+      <formula>"No"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M2:M200">
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="0">
+      <formula>"Applied"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="1">
+      <formula>"Drafted (not applied)"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" dxfId="3">
+      <formula>"Destroyed"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L2:L200">
+    <cfRule type="cellIs" priority="6" operator="equal" dxfId="1">
+      <formula>"Not verified"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="7" operator="equal" dxfId="0">
+      <formula>"Verified"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="D2:D200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Low,Medium,High"</formula1>
+    <dataValidation sqref="M2:M200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Drafted (not applied),Planned,Applied,Destroyed"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3295,170 +6515,1415 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:L24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="70" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>Document</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="B1" s="11" t="inlineStr">
         <is>
-          <t>Version</t>
+          <t>Script</t>
         </is>
       </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Purpose</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
         <is>
-          <t>Type</t>
+          <t>Phase</t>
         </is>
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Summary</t>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>AWS services / permissions</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>Inputs</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Outputs</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>Serves (P#)</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="K1" s="11" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="L1" s="11" t="inlineStr">
+        <is>
+          <t>Path</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="13" t="inlineStr">
-        <is>
-          <t>DESIGN.md</t>
-        </is>
-      </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>0.1.0</t>
-        </is>
-      </c>
-      <c r="C2" s="14" t="n">
-        <v>46297</v>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>Initial draft</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>Base plan: architecture, components, cost model, roadmap</t>
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>PY-01</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>build_lambda_package.py</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Build a reproducible arm64 Lambda zip (pip --platform manylinux2014_aarch64) and its SHA-256</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Manual / CI</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>src/, requirements.txt</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>dist/app.zip + sha256</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J2" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K2" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="inlineStr">
+        <is>
+          <t>scripts/build_lambda_package.py</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
-        <is>
-          <t>DESIGN.md</t>
-        </is>
-      </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>0.1.1</t>
-        </is>
-      </c>
-      <c r="C3" s="14" t="n">
-        <v>46297</v>
-      </c>
-      <c r="D3" s="13" t="inlineStr">
-        <is>
-          <t>Patch</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
-        <is>
-          <t>Budget set to ₹5,000/month; budget fit added</t>
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>PY-02</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>db_migrate.py</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Apply SQL migrations via RDS Data API; CREATE EXTENSION vector; create least-privilege app user + its secret</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Manual / CI after deploy</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>rds-data, secretsmanager</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>migrations/*.sql</t>
+        </is>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>schema_version table</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="inlineStr">
+        <is>
+          <t>scripts/db_migrate.py</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
-        <is>
-          <t>DESIGN.md</t>
-        </is>
-      </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>0.1.2</t>
-        </is>
-      </c>
-      <c r="C4" s="14" t="n">
-        <v>46297</v>
-      </c>
-      <c r="D4" s="13" t="inlineStr">
-        <is>
-          <t>Patch</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
-        <is>
-          <t>FigJam board link; data exit X8 (Figma)</t>
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>PY-03</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>set_secret.py</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Store a secret value from a hidden prompt or file (never a CLI arg); verify KMS key; never echo</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>secretsmanager, kms</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>secret name</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>secret version id</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="inlineStr">
+        <is>
+          <t>scripts/set_secret.py</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
-        <is>
-          <t>DESIGN.md</t>
-        </is>
-      </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>0.1.3</t>
-        </is>
-      </c>
-      <c r="C5" s="14" t="n">
-        <v>46297</v>
-      </c>
-      <c r="D5" s="13" t="inlineStr">
-        <is>
-          <t>Patch</t>
-        </is>
-      </c>
-      <c r="E5" s="13" t="inlineStr">
-        <is>
-          <t>Diagram images added (docs/diagrams/: jpg, svg, mmd)</t>
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>PY-04</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>bedrock_smoke_test.py</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Confirm India-profile model access, latency and token cost for a test prompt</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>bedrock:InvokeModel</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>model ids</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>latency / cost report</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>scripts/bedrock_smoke_test.py</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
-        <is>
-          <t>Tracker</t>
-        </is>
-      </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>1.1</t>
-        </is>
-      </c>
-      <c r="C6" s="14" t="n">
-        <v>46297</v>
-      </c>
-      <c r="D6" s="13" t="inlineStr">
-        <is>
-          <t>Patch</t>
-        </is>
-      </c>
-      <c r="E6" s="13" t="inlineStr">
-        <is>
-          <t>Costs verified against AWS Price List API (ap-south-1); FX 96.12; I-3 closed</t>
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>PY-05</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>aurora_wake_check.py</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Measure Aurora resume time after auto-pause; tune retry/backoff</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>rds-data</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>cluster ARN</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>resume seconds</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="inlineStr">
+        <is>
+          <t>scripts/aurora_wake_check.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>PY-06</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>secret_scan.py</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Pre-commit/CI guard for the public repo: gitleaks + regex for account IDs, IPs, keys</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>pre-commit / CI</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>staged files</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>pass / fail</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L7" s="12" t="inlineStr">
+        <is>
+          <t>scripts/secret_scan.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>PY-07</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>bootstrap_owner.py</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Create the single owner row + one-time passkey registration code (shown once over SSM)</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Manual, once</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>rds-data, secretsmanager</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>registration code</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="inlineStr">
+        <is>
+          <t>scripts/bootstrap_owner.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>PY-08</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>reminder_scheduler.py (app module)</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Create/delete one-time EventBridge schedules for reminders (no polling)</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Called by API</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>scheduler, iam:PassRole</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>reminder</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>schedule ARN</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>src/weekend/reminders.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>PY-09</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>tailscale_authkey_rotate.py</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Create a new tagged Tailscale auth key via API and store it in Secrets Manager before expiry</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Tailscale API, secretsmanager</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>new secret version</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L10" s="12" t="inlineStr">
+        <is>
+          <t>scripts/tailscale_authkey_rotate.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>PY-10</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>voice_benchmark.py</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Benchmark STT/TTS options (on-device, Transcribe, Polly, local) for latency and ₹/minute</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>transcribe, polly</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>sample audio</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>benchmark table</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L11" s="12" t="inlineStr">
+        <is>
+          <t>scripts/voice_benchmark.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>PY-11</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>data_export.py</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Export all owner data to an encrypted archive in S3</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Worker 03:30 IST + on demand</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>rds-data, s3, kms</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>s3://…/daily/</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>P6, P10</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K12" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L12" s="12" t="inlineStr">
+        <is>
+          <t>scripts/data_export.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>PY-12</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>retention_cleanup.py</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Delete data past its retention per table; write audit entries</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Worker 03:00 IST</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>rds-data</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>retention table</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>deleted counts</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>P5, P8</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>scripts/retention_cleanup.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>PY-13</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>delete_all_data.py</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>'Forget everything': purge DB rows + S3 objects (respecting Object Lock) with double confirmation</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>rds-data, s3</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>confirmation phrase</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>purge report</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K14" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L14" s="12" t="inlineStr">
+        <is>
+          <t>scripts/delete_all_data.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>PY-14</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>audit_verify.py</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Verify the audit_log hash chain against S3 Object Lock copies</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Weekly / manual</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>rds-data, s3</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>pass / fail</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L15" s="12" t="inlineStr">
+        <is>
+          <t>scripts/audit_verify.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>PY-15</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>tailnet_check.py</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Check Tailscale devices/ACLs: only owner devices + tag:weekend; alert on a new device</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Tailscale API</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>P1, P9</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L16" s="12" t="inlineStr">
+        <is>
+          <t>scripts/tailnet_check.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>PY-16</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>restore_drill.py</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Restore latest snapshot to a temporary cluster, run integrity checks, record result, delete the temp cluster</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>rds, rds-data</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>snapshot id</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>drill record</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L17" s="12" t="inlineStr">
+        <is>
+          <t>scripts/restore_drill.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>PY-17</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>healthcheck.py</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Synthetic check via the tailnet: login page, API health, Bedrock call (runs daily, not per-minute, so Aurora can pause)</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Daily 09:00 IST / manual</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>None (tailnet)</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>status report</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L18" s="12" t="inlineStr">
+        <is>
+          <t>scripts/healthcheck.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>PY-18</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>cost_report.py</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Month-to-date + forecast cost vs ₹5,000 using live FX; append to tracker</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Daily / manual</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>ce:GetCostAndUsage, ce:GetCostForecast</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>INR report</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L19" s="12" t="inlineStr">
+        <is>
+          <t>scripts/cost_report.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>PY-19</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>price_check.py</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Pull AWS Price List (ap-south-1) for every tracked resource; flag changes; update Resources sheet</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>None (public price list)</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Resources sheet</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>updated prices</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L20" s="12" t="inlineStr">
+        <is>
+          <t>scripts/price_check.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>PY-20</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>fx_rate_update.py</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Fetch USD/INR from 3 sources, take the median, update Cost!B15 with date and sources</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>Daily / manual</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>None (public APIs)</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>rate + sources</t>
+        </is>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L21" s="12" t="inlineStr">
+        <is>
+          <t>scripts/fx_rate_update.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>PY-21</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>tracker_sync.py</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Sync tracker tables (tasks, issues, decisions) with PROJECT_MEMORY.md</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>tracker + memory</t>
+        </is>
+      </c>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>diff report</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L22" s="12" t="inlineStr">
+        <is>
+          <t>scripts/tracker_sync.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>Standards: Python 3.12+ (Lambda runtime python3.14), type hints, logging (not print), argparse, explicit non-zero exits, pytest tests, ruff/black. Secrets only from Secrets Manager.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E5"/>
+  <autoFilter ref="A1:L22"/>
+  <conditionalFormatting sqref="K2:K200">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"In progress"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
+      <formula>"Planned"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="K2:K200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Planned,In progress,Done,Dropped"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(infra): apply adversarial review findings before first apply
- entry_node: split Function URL IAM into InvokeFunctionUrl (FunctionUrlAuthType)
  and InvokeFunction (InvokedViaFunctionUrl), per AWS Lambda urls-auth docs
- entry_node: user_data waits (max ~20 min) for the Tailscale auth key instead of
  failing on first boot; README run order creates secrets before the instance
- app: Function URL BUFFERED (Python has no native response streaming)
- app/backup: worker writes only to daily/monthly/audit prefixes; per-object
  Object Lock for monthly/ (365 d) and audit/ (730 d); 30-day noncurrent recovery
- tailscale/policy.hujson: owner-only grant to tag:weekend:443 (P1)
- README: Bedrock model enablement step, plans outside the repo, P6 purge,
  18% GST in the cost estimate; .gitignore ignores tfplan files
- tracker v1.3: GST line, issues I-9..I-12

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/Weekend2.0_Tracker.xlsx
+++ b/tracking/Weekend2.0_Tracker.xlsx
@@ -828,7 +828,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1012,6 +1012,31 @@
       <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Resources sheet (39 lines, E2 Terraform) + Automation Scripts sheet (21 scripts); tasks T-016–T-019; issues I-7, I-8</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="13" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="C8" s="14" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D8" s="13" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="E8" s="13" t="inlineStr">
+        <is>
+          <t>Terraform review fixes: 18% GST line in Resources; Function URL BUFFERED; per-object Object Lock; issues I-9–I-12</t>
         </is>
       </c>
     </row>
@@ -2987,7 +3012,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3285,6 +3310,130 @@
         <v>46297</v>
       </c>
       <c r="G9" s="14" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>I-9</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Owner Gmail visible in the first two public commits</t>
+        </is>
+      </c>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D10" s="13" t="inlineStr">
+        <is>
+          <t>Accept, or rewrite history + force-push (needs a checkpoint)</t>
+        </is>
+      </c>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G10" s="14" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>I-10</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>Local Terraform is 1.5.7; infra needs &gt;= 1.16</t>
+        </is>
+      </c>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D11" s="13" t="inlineStr">
+        <is>
+          <t>brew install hashicorp/tap/terraform (T-019)</t>
+        </is>
+      </c>
+      <c r="E11" s="13" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F11" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G11" s="14" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>I-11</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>With 18% GST the expected bill is ≈ ₹4,854 (97% of ₹5,000); headroom ≈ ₹146</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D12" s="13" t="inlineStr">
+        <is>
+          <t>Confirm billing entity; consider Aurora max 1 ACU or dropping public IPv4</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F12" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G12" s="14" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>I-12</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Python Lambda cannot stream replies natively; Function URL set to BUFFERED</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Decide in Phase 1: Lambda Web Adapter (stream) or keep buffered</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F13" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G13" s="14" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G7"/>
@@ -5214,7 +5363,7 @@
       </c>
       <c r="H22" s="12" t="inlineStr">
         <is>
-          <t>AWS_IAM auth; RESPONSE_STREAM</t>
+          <t>AWS_IAM auth; BUFFERED (Python cannot stream natively; Web Adapter = Phase 1)</t>
         </is>
       </c>
       <c r="I22" s="26" t="n">
@@ -6189,7 +6338,7 @@
       </c>
       <c r="H37" s="12" t="inlineStr">
         <is>
-          <t>Object Lock governance 35 d; SSE-KMS; versioning; TLS-only; lifecycle</t>
+          <t>Object Lock governance 35 d default; monthly/ 365 d + audit/ 730 d per object; SSE-KMS; versioning; TLS-only; lifecycle</t>
         </is>
       </c>
       <c r="I37" s="26" t="n">
@@ -6413,18 +6562,86 @@
         <v>1</v>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>GST</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="inlineStr">
+        <is>
+          <t>(no resource — tax on the AWS bill)</t>
+        </is>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>GST (IGST 18%)</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>AWS India (AISPL) invoice</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F41" s="12" t="inlineStr">
+        <is>
+          <t>India</t>
+        </is>
+      </c>
+      <c r="G41" s="12" t="inlineStr">
+        <is>
+          <t>Tax added to every AWS charge</t>
+        </is>
+      </c>
+      <c r="H41" s="12" t="inlineStr">
+        <is>
+          <t>18% of lines 1–39; assumes AISPL billing (check Billing → Account)</t>
+        </is>
+      </c>
+      <c r="I41" s="26">
+        <f>ROUND(SUM(I2:I40)*0.18,2)</f>
+        <v/>
+      </c>
+      <c r="J41" s="27">
+        <f>I41*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="K41" s="12" t="inlineStr">
+        <is>
+          <t>AISPL charges 18% GST on AWS services</t>
+        </is>
+      </c>
+      <c r="L41" s="13" t="inlineStr">
+        <is>
+          <t>Assumption (confirm entity)</t>
+        </is>
+      </c>
+      <c r="M41" s="13" t="inlineStr">
+        <is>
+          <t>Applies on apply</t>
+        </is>
+      </c>
+      <c r="N41" s="12" t="n">
+        <v>1</v>
+      </c>
+    </row>
     <row r="42">
       <c r="H42" s="3" t="inlineStr">
         <is>
-          <t>Total per month (expected use)</t>
+          <t>Total per month incl. 18% GST (expected use)</t>
         </is>
       </c>
       <c r="I42" s="33">
-        <f>SUM(I2:I40)</f>
+        <f>SUM(I2:I41)</f>
         <v/>
       </c>
       <c r="J42" s="34">
-        <f>SUM(J2:J40)</f>
+        <f>SUM(J2:J41)</f>
         <v/>
       </c>
     </row>
@@ -6467,7 +6684,7 @@
     <row r="47">
       <c r="A47" s="23" t="inlineStr">
         <is>
-          <t>Design: D1 option E2 (revised) — PROVISIONAL until D1 is decided. Source: infra/ (Terraform 1.16.5 / AWS provider 6.67.0, validated 2026-10-02). INR uses Cost!B15. Aurora hours are the main uncertainty.</t>
+          <t>Design: D1 option E2 (revised) — PROVISIONAL until D1 is decided. Source: infra/ (Terraform 1.16.5 / AWS provider 6.67.0, validated 2026-10-02). INR uses Cost!B15. Aurora hours are the main uncertainty. Review 2026-10-02: GST line added (tracker v1.3); total now includes 18% GST.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(infra): add dev environment (free-tier sizing, destroyable)
- envs/dev: same modules as prod; weekend2-dev prefix, VPC 10.30.0.0/16
  - entry node t4g.small (EC2 T4g free trial until 2026-12-31), optional via entry_node_enabled
  - Aurora 0-1 ACU, 1-day backups, no deletion protection / final snapshot
  - KMS 7-day window, secrets recovery 0, backup bucket force_destroy + 1-day lock
  - no Google connector secret, 3-day logs, Haiku for both model slots, USD 12 budget
- modules: new opt-in knobs (kms deletion_window_in_days, secrets recovery_window_in_days,
  database deletion_protection/skip_final_snapshot, backup force_destroy); prod defaults unchanged
- tailscale policy: tag:weekend-dev, dev cannot reach prod; real copy *.local.hujson git-ignored
- README: dev table, cost (~INR 1,042/month incl. GST), run order, smoke tests, teardown
- tracker v1.4: Dev env sheet, T-020/T-021, I-13..I-15

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/Weekend2.0_Tracker.xlsx
+++ b/tracking/Weekend2.0_Tracker.xlsx
@@ -15,9 +15,10 @@
     <sheet name="Issues" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Cost" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Resources" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Automation Scripts" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Approvals" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Doc versions" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Dev env" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Automation Scripts" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Approvals" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Doc versions" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Phases'!$A$1:$J$8</definedName>
@@ -26,9 +27,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Issues'!$A$1:$G$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Cost'!$A$1:$F$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Resources'!$A$1:$N$40</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Automation Scripts'!$A$1:$L$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Approvals'!$A$1:$E$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Doc versions'!$A$1:$E$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Automation Scripts'!$A$1:$L$22</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Approvals'!$A$1:$E$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Doc versions'!$A$1:$E$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -45,7 +46,7 @@
     <numFmt numFmtId="169" formatCode="₹#,##0"/>
     <numFmt numFmtId="170" formatCode="$#,##0.000;($#,##0.000);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -81,6 +82,11 @@
       <name val="Arial"/>
       <i val="1"/>
       <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="4">
@@ -127,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -189,6 +195,8 @@
     <xf numFmtId="169" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -749,6 +757,1425 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:L24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="58" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" s="11" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="C1" s="11" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="D1" s="11" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
+      <c r="E1" s="11" t="inlineStr">
+        <is>
+          <t>Trigger</t>
+        </is>
+      </c>
+      <c r="F1" s="11" t="inlineStr">
+        <is>
+          <t>AWS services / permissions</t>
+        </is>
+      </c>
+      <c r="G1" s="11" t="inlineStr">
+        <is>
+          <t>Inputs</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
+          <t>Outputs</t>
+        </is>
+      </c>
+      <c r="I1" s="11" t="inlineStr">
+        <is>
+          <t>Serves (P#)</t>
+        </is>
+      </c>
+      <c r="J1" s="11" t="inlineStr">
+        <is>
+          <t>Priority</t>
+        </is>
+      </c>
+      <c r="K1" s="11" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="L1" s="11" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>PY-01</t>
+        </is>
+      </c>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>build_lambda_package.py</t>
+        </is>
+      </c>
+      <c r="C2" s="12" t="inlineStr">
+        <is>
+          <t>Build a reproducible arm64 Lambda zip (pip --platform manylinux2014_aarch64) and its SHA-256</t>
+        </is>
+      </c>
+      <c r="D2" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E2" s="12" t="inlineStr">
+        <is>
+          <t>Manual / CI</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G2" s="12" t="inlineStr">
+        <is>
+          <t>src/, requirements.txt</t>
+        </is>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>dist/app.zip + sha256</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J2" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K2" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L2" s="12" t="inlineStr">
+        <is>
+          <t>scripts/build_lambda_package.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="inlineStr">
+        <is>
+          <t>PY-02</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>db_migrate.py</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>Apply SQL migrations via RDS Data API; CREATE EXTENSION vector; create least-privilege app user + its secret</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
+        <is>
+          <t>Manual / CI after deploy</t>
+        </is>
+      </c>
+      <c r="F3" s="12" t="inlineStr">
+        <is>
+          <t>rds-data, secretsmanager</t>
+        </is>
+      </c>
+      <c r="G3" s="12" t="inlineStr">
+        <is>
+          <t>migrations/*.sql</t>
+        </is>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>schema_version table</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="J3" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L3" s="12" t="inlineStr">
+        <is>
+          <t>scripts/db_migrate.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>PY-03</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>set_secret.py</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Store a secret value from a hidden prompt or file (never a CLI arg); verify KMS key; never echo</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>secretsmanager, kms</t>
+        </is>
+      </c>
+      <c r="G4" s="12" t="inlineStr">
+        <is>
+          <t>secret name</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>secret version id</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="J4" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K4" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L4" s="12" t="inlineStr">
+        <is>
+          <t>scripts/set_secret.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>PY-04</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>bedrock_smoke_test.py</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Confirm India-profile model access, latency and token cost for a test prompt</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>bedrock:InvokeModel</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>model ids</t>
+        </is>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>latency / cost report</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L5" s="12" t="inlineStr">
+        <is>
+          <t>scripts/bedrock_smoke_test.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="inlineStr">
+        <is>
+          <t>PY-05</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>aurora_wake_check.py</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>Measure Aurora resume time after auto-pause; tune retry/backoff</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>rds-data</t>
+        </is>
+      </c>
+      <c r="G6" s="12" t="inlineStr">
+        <is>
+          <t>cluster ARN</t>
+        </is>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>resume seconds</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J6" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L6" s="12" t="inlineStr">
+        <is>
+          <t>scripts/aurora_wake_check.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="inlineStr">
+        <is>
+          <t>PY-06</t>
+        </is>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>secret_scan.py</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>Pre-commit/CI guard for the public repo: gitleaks + regex for account IDs, IPs, keys</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>pre-commit / CI</t>
+        </is>
+      </c>
+      <c r="F7" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G7" s="12" t="inlineStr">
+        <is>
+          <t>staged files</t>
+        </is>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>pass / fail</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="J7" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L7" s="12" t="inlineStr">
+        <is>
+          <t>scripts/secret_scan.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="inlineStr">
+        <is>
+          <t>PY-07</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>bootstrap_owner.py</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Create the single owner row + one-time passkey registration code (shown once over SSM)</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>Manual, once</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="inlineStr">
+        <is>
+          <t>rds-data, secretsmanager</t>
+        </is>
+      </c>
+      <c r="G8" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>registration code</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="J8" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L8" s="12" t="inlineStr">
+        <is>
+          <t>scripts/bootstrap_owner.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>PY-08</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>reminder_scheduler.py (app module)</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>Create/delete one-time EventBridge schedules for reminders (no polling)</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Called by API</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="inlineStr">
+        <is>
+          <t>scheduler, iam:PassRole</t>
+        </is>
+      </c>
+      <c r="G9" s="12" t="inlineStr">
+        <is>
+          <t>reminder</t>
+        </is>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>schedule ARN</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>P5</t>
+        </is>
+      </c>
+      <c r="J9" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K9" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L9" s="12" t="inlineStr">
+        <is>
+          <t>src/weekend/reminders.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>PY-09</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>tailscale_authkey_rotate.py</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>Create a new tagged Tailscale auth key via API and store it in Secrets Manager before expiry</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="inlineStr">
+        <is>
+          <t>Tailscale API, secretsmanager</t>
+        </is>
+      </c>
+      <c r="G10" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>new secret version</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="J10" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L10" s="12" t="inlineStr">
+        <is>
+          <t>scripts/tailscale_authkey_rotate.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>PY-10</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>voice_benchmark.py</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>Benchmark STT/TTS options (on-device, Transcribe, Polly, local) for latency and ₹/minute</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="inlineStr">
+        <is>
+          <t>transcribe, polly</t>
+        </is>
+      </c>
+      <c r="G11" s="12" t="inlineStr">
+        <is>
+          <t>sample audio</t>
+        </is>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
+        <is>
+          <t>benchmark table</t>
+        </is>
+      </c>
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>P7</t>
+        </is>
+      </c>
+      <c r="J11" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L11" s="12" t="inlineStr">
+        <is>
+          <t>scripts/voice_benchmark.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="inlineStr">
+        <is>
+          <t>PY-11</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>data_export.py</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>Export all owner data to an encrypted archive in S3</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>Worker 03:30 IST + on demand</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="inlineStr">
+        <is>
+          <t>rds-data, s3, kms</t>
+        </is>
+      </c>
+      <c r="G12" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>s3://…/daily/</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>P6, P10</t>
+        </is>
+      </c>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K12" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L12" s="12" t="inlineStr">
+        <is>
+          <t>scripts/data_export.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>PY-12</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>retention_cleanup.py</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Delete data past its retention per table; write audit entries</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Worker 03:00 IST</t>
+        </is>
+      </c>
+      <c r="F13" s="12" t="inlineStr">
+        <is>
+          <t>rds-data</t>
+        </is>
+      </c>
+      <c r="G13" s="12" t="inlineStr">
+        <is>
+          <t>retention table</t>
+        </is>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>deleted counts</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>P5, P8</t>
+        </is>
+      </c>
+      <c r="J13" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L13" s="12" t="inlineStr">
+        <is>
+          <t>scripts/retention_cleanup.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>PY-13</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>delete_all_data.py</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>'Forget everything': purge DB rows + S3 objects (respecting Object Lock) with double confirmation</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F14" s="12" t="inlineStr">
+        <is>
+          <t>rds-data, s3</t>
+        </is>
+      </c>
+      <c r="G14" s="12" t="inlineStr">
+        <is>
+          <t>confirmation phrase</t>
+        </is>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>purge report</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>P6</t>
+        </is>
+      </c>
+      <c r="J14" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K14" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L14" s="12" t="inlineStr">
+        <is>
+          <t>scripts/delete_all_data.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>PY-14</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>audit_verify.py</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Verify the audit_log hash chain against S3 Object Lock copies</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Weekly / manual</t>
+        </is>
+      </c>
+      <c r="F15" s="12" t="inlineStr">
+        <is>
+          <t>rds-data, s3</t>
+        </is>
+      </c>
+      <c r="G15" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>pass / fail</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>P8</t>
+        </is>
+      </c>
+      <c r="J15" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L15" s="12" t="inlineStr">
+        <is>
+          <t>scripts/audit_verify.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>PY-15</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>tailnet_check.py</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Check Tailscale devices/ACLs: only owner devices + tag:weekend; alert on a new device</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Daily</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="inlineStr">
+        <is>
+          <t>Tailscale API</t>
+        </is>
+      </c>
+      <c r="G16" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>report</t>
+        </is>
+      </c>
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>P1, P9</t>
+        </is>
+      </c>
+      <c r="J16" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L16" s="12" t="inlineStr">
+        <is>
+          <t>scripts/tailnet_check.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>PY-16</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>restore_drill.py</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>Restore latest snapshot to a temporary cluster, run integrity checks, record result, delete the temp cluster</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Quarterly</t>
+        </is>
+      </c>
+      <c r="F17" s="12" t="inlineStr">
+        <is>
+          <t>rds, rds-data</t>
+        </is>
+      </c>
+      <c r="G17" s="12" t="inlineStr">
+        <is>
+          <t>snapshot id</t>
+        </is>
+      </c>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>drill record</t>
+        </is>
+      </c>
+      <c r="I17" s="12" t="inlineStr">
+        <is>
+          <t>P10</t>
+        </is>
+      </c>
+      <c r="J17" s="13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L17" s="12" t="inlineStr">
+        <is>
+          <t>scripts/restore_drill.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>PY-17</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>healthcheck.py</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Synthetic check via the tailnet: login page, API health, Bedrock call (runs daily, not per-minute, so Aurora can pause)</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Daily 09:00 IST / manual</t>
+        </is>
+      </c>
+      <c r="F18" s="12" t="inlineStr">
+        <is>
+          <t>None (tailnet)</t>
+        </is>
+      </c>
+      <c r="G18" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H18" s="12" t="inlineStr">
+        <is>
+          <t>status report</t>
+        </is>
+      </c>
+      <c r="I18" s="12" t="inlineStr">
+        <is>
+          <t>P9</t>
+        </is>
+      </c>
+      <c r="J18" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K18" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L18" s="12" t="inlineStr">
+        <is>
+          <t>scripts/healthcheck.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>PY-18</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>cost_report.py</t>
+        </is>
+      </c>
+      <c r="C19" s="12" t="inlineStr">
+        <is>
+          <t>Month-to-date + forecast cost vs ₹5,000 using live FX; append to tracker</t>
+        </is>
+      </c>
+      <c r="D19" s="12" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="E19" s="12" t="inlineStr">
+        <is>
+          <t>Daily / manual</t>
+        </is>
+      </c>
+      <c r="F19" s="12" t="inlineStr">
+        <is>
+          <t>ce:GetCostAndUsage, ce:GetCostForecast</t>
+        </is>
+      </c>
+      <c r="G19" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H19" s="12" t="inlineStr">
+        <is>
+          <t>INR report</t>
+        </is>
+      </c>
+      <c r="I19" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J19" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L19" s="12" t="inlineStr">
+        <is>
+          <t>scripts/cost_report.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>PY-19</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>price_check.py</t>
+        </is>
+      </c>
+      <c r="C20" s="12" t="inlineStr">
+        <is>
+          <t>Pull AWS Price List (ap-south-1) for every tracked resource; flag changes; update Resources sheet</t>
+        </is>
+      </c>
+      <c r="D20" s="12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F20" s="12" t="inlineStr">
+        <is>
+          <t>None (public price list)</t>
+        </is>
+      </c>
+      <c r="G20" s="12" t="inlineStr">
+        <is>
+          <t>Resources sheet</t>
+        </is>
+      </c>
+      <c r="H20" s="12" t="inlineStr">
+        <is>
+          <t>updated prices</t>
+        </is>
+      </c>
+      <c r="I20" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J20" s="13" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L20" s="12" t="inlineStr">
+        <is>
+          <t>scripts/price_check.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>PY-20</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>fx_rate_update.py</t>
+        </is>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Fetch USD/INR from 3 sources, take the median, update Cost!B15 with date and sources</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>Daily / manual</t>
+        </is>
+      </c>
+      <c r="F21" s="12" t="inlineStr">
+        <is>
+          <t>None (public APIs)</t>
+        </is>
+      </c>
+      <c r="G21" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H21" s="12" t="inlineStr">
+        <is>
+          <t>rate + sources</t>
+        </is>
+      </c>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J21" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L21" s="12" t="inlineStr">
+        <is>
+          <t>scripts/fx_rate_update.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>PY-21</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>tracker_sync.py</t>
+        </is>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Sync tracker tables (tasks, issues, decisions) with PROJECT_MEMORY.md</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F22" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr">
+        <is>
+          <t>tracker + memory</t>
+        </is>
+      </c>
+      <c r="H22" s="12" t="inlineStr">
+        <is>
+          <t>diff report</t>
+        </is>
+      </c>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J22" s="13" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>Planned</t>
+        </is>
+      </c>
+      <c r="L22" s="12" t="inlineStr">
+        <is>
+          <t>scripts/tracker_sync.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>Standards: Python 3.12+ (Lambda runtime python3.14), type hints, logging (not print), argparse, explicit non-zero exits, pytest tests, ruff/black. Secrets only from Secrets Manager.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:L22"/>
+  <conditionalFormatting sqref="K2:K200">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Done"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"In progress"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
+      <formula>"Planned"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="K2:K200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Planned,In progress,Done,Dropped"</formula1>
+    </dataValidation>
+    <dataValidation sqref="J2:J200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"High,Medium,Low"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -822,13 +2249,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1037,6 +2464,31 @@
       <c r="E8" s="13" t="inlineStr">
         <is>
           <t>Terraform review fixes: 18% GST line in Resources; Function URL BUFFERED; per-object Object Lock; issues I-9–I-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="C9" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Dev env sheet (envs/dev, free-tier sizing, ≈ ₹1,042/month incl. GST); tasks T-020, T-021; issues I-13–I-15</t>
         </is>
       </c>
     </row>
@@ -1052,7 +2504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D50"/>
+  <dimension ref="A1:D52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1639,6 +3091,28 @@
       </c>
       <c r="B50" s="5">
         <f>COUNTIFS('Automation Scripts'!$J$2:$J$200,"High",'Automation Scripts'!$K$2:$K$200,"&lt;&gt;Done")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>Dev estimated cost (₹/month)</t>
+        </is>
+      </c>
+      <c r="B51" s="32">
+        <f>'Dev env'!G19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>Dev + prod within budget?</t>
+        </is>
+      </c>
+      <c r="B52" s="5">
+        <f>'Dev env'!G23</f>
         <v/>
       </c>
     </row>
@@ -2022,7 +3496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -2721,6 +4195,74 @@
       <c r="G20" s="14" t="n"/>
       <c r="H20" s="14" t="n"/>
       <c r="I20" s="13" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>T-020</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C21" s="12" t="inlineStr">
+        <is>
+          <t>Deploy dev environment (infra/envs/dev) — files ready; owner runs plan/apply after security checkpoint</t>
+        </is>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F21" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G21" s="16" t="n"/>
+      <c r="H21" s="16" t="n"/>
+      <c r="I21" s="12" t="inlineStr">
+        <is>
+          <t>infra/README.md → Dev run order</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>T-021</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="C22" s="12" t="inlineStr">
+        <is>
+          <t>Fill infra/tailscale/policy.local.hujson (git-ignored) and apply in Tailscale admin console</t>
+        </is>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F22" s="16" t="n"/>
+      <c r="G22" s="16" t="n"/>
+      <c r="H22" s="16" t="n"/>
+      <c r="I22" s="12" t="inlineStr">
+        <is>
+          <t>Before the dev entry node first boots</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:I16"/>
@@ -3012,7 +4554,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3434,6 +4976,99 @@
         <v>46297</v>
       </c>
       <c r="G13" s="14" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>I-13</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Dev (≈ ₹1,042) + prod (≈ ₹4,855) together ≈ ₹5,900 — over the ₹5,000 budget</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Destroy dev (or stop its node) before prod goes live</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F14" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G14" s="16" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>I-14</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>EC2 T4g free trial (t4g.small) ends 2026-12-31; dev node then becomes paid</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Set entry_node_instance_type = "t4g.nano" in envs/dev before 2026-12-31</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F15" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G15" s="16" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>I-15</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>On an AWS Free plan account, Claude models on Bedrock (Marketplace) may be blocked — Not verified</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Check plan (Billing → Free Tier); upgrade to Paid plan if model enablement fails</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F16" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="G16" s="16" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G7"/>
@@ -6732,1415 +8367,982 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:J30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="58" customWidth="1" min="3" max="3"/>
-    <col width="7" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="11" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>#</t>
         </is>
       </c>
       <c r="B1" s="11" t="inlineStr">
         <is>
-          <t>Script</t>
+          <t>Resource</t>
         </is>
       </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>Purpose</t>
+          <t>Name (weekend2-dev-*)</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
         <is>
-          <t>Phase</t>
+          <t>Key settings</t>
         </is>
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Trigger</t>
+          <t>Free tier / trial</t>
         </is>
       </c>
       <c r="F1" s="11" t="inlineStr">
         <is>
-          <t>AWS services / permissions</t>
+          <t>USD / month</t>
         </is>
       </c>
       <c r="G1" s="11" t="inlineStr">
         <is>
-          <t>Inputs</t>
+          <t>INR / month</t>
         </is>
       </c>
       <c r="H1" s="11" t="inlineStr">
         <is>
-          <t>Outputs</t>
+          <t>Price basis / source</t>
         </is>
       </c>
       <c r="I1" s="11" t="inlineStr">
         <is>
-          <t>Serves (P#)</t>
+          <t>Verified?</t>
         </is>
       </c>
       <c r="J1" s="11" t="inlineStr">
         <is>
-          <t>Priority</t>
-        </is>
-      </c>
-      <c r="K1" s="11" t="inlineStr">
-        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="L1" s="11" t="inlineStr">
-        <is>
-          <t>Path</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
-        <is>
-          <t>PY-01</t>
-        </is>
+      <c r="A2" s="12" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="12" t="inlineStr">
         <is>
-          <t>build_lambda_package.py</t>
+          <t>Network (VPC, 3 subnets, IGW, 2 route tables, SGs)</t>
         </is>
       </c>
       <c r="C2" s="12" t="inlineStr">
         <is>
-          <t>Build a reproducible arm64 Lambda zip (pip --platform manylinux2014_aarch64) and its SHA-256</t>
+          <t>weekend2-dev-vpc …</t>
         </is>
       </c>
       <c r="D2" s="12" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>10.30.0.0/16; no NAT; no inbound rules</t>
         </is>
       </c>
       <c r="E2" s="12" t="inlineStr">
         <is>
-          <t>Manual / CI</t>
-        </is>
-      </c>
-      <c r="F2" s="12" t="inlineStr">
+          <t>No charge</t>
+        </is>
+      </c>
+      <c r="F2" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="12">
+        <f>F2*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H2" s="12" t="inlineStr">
+        <is>
+          <t>No charge for VPC objects</t>
+        </is>
+      </c>
+      <c r="I2" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="J2" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>KMS CMK</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>alias/weekend2-dev-data</t>
+        </is>
+      </c>
+      <c r="D3" s="12" t="inlineStr">
+        <is>
+          <t>Rotation 365 d; 7-day deletion window</t>
+        </is>
+      </c>
+      <c r="E3" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G2" s="12" t="inlineStr">
-        <is>
-          <t>src/, requirements.txt</t>
-        </is>
-      </c>
-      <c r="H2" s="12" t="inlineStr">
-        <is>
-          <t>dist/app.zip + sha256</t>
-        </is>
-      </c>
-      <c r="I2" s="12" t="inlineStr">
+      <c r="F3" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" s="12">
+        <f>F3*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H3" s="12" t="inlineStr">
+        <is>
+          <t>$1/key-month (AWS Price List API ap-south-1 2026-09-11)</t>
+        </is>
+      </c>
+      <c r="I3" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="J3" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-dev/tailscale/authkey</t>
+        </is>
+      </c>
+      <c r="D4" s="12" t="inlineStr">
+        <is>
+          <t>KMS; recovery window 0 (dev)</t>
+        </is>
+      </c>
+      <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G4" s="12">
+        <f>F4*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>$0.40/secret-month</t>
+        </is>
+      </c>
+      <c r="I4" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="J4" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Secret</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-dev/app/session-signing-key</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>KMS</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G5" s="12">
+        <f>F5*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>$0.40/secret-month</t>
+        </is>
+      </c>
+      <c r="I5" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="J5" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Secret (RDS-managed)</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>rds!cluster-&lt;id&gt;</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Aurora master password, rotated by RDS</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G6" s="12">
+        <f>F6*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>$0.40/secret-month</t>
+        </is>
+      </c>
+      <c r="I6" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="J6" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="12" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="12" t="inlineStr">
+        <is>
+          <t>Aurora PostgreSQL Serverless v2 (compute)</t>
+        </is>
+      </c>
+      <c r="C7" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-dev-aurora</t>
+        </is>
+      </c>
+      <c r="D7" s="12" t="inlineStr">
+        <is>
+          <t>0–1 ACU; pause after 300 s; Data API; no deletion protection; 1-day backups</t>
+        </is>
+      </c>
+      <c r="E7" s="12" t="n"/>
+      <c r="F7" s="12">
+        <f>ROUND($F$26*0.5*0.18,2)</f>
+        <v/>
+      </c>
+      <c r="G7" s="12">
+        <f>F7*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>$0.18/ACU-h × 0.5 ACU × active hours (F26)</t>
+        </is>
+      </c>
+      <c r="I7" s="12" t="inlineStr">
+        <is>
+          <t>Rate verified; hours estimate</t>
+        </is>
+      </c>
+      <c r="J7" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="12" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Aurora storage + I/O</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J2" s="13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K2" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L2" s="12" t="inlineStr">
-        <is>
-          <t>scripts/build_lambda_package.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="12" t="inlineStr">
-        <is>
-          <t>PY-02</t>
-        </is>
-      </c>
-      <c r="B3" s="12" t="inlineStr">
-        <is>
-          <t>db_migrate.py</t>
-        </is>
-      </c>
-      <c r="C3" s="12" t="inlineStr">
-        <is>
-          <t>Apply SQL migrations via RDS Data API; CREATE EXTENSION vector; create least-privilege app user + its secret</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E3" s="12" t="inlineStr">
-        <is>
-          <t>Manual / CI after deploy</t>
-        </is>
-      </c>
-      <c r="F3" s="12" t="inlineStr">
-        <is>
-          <t>rds-data, secretsmanager</t>
-        </is>
-      </c>
-      <c r="G3" s="12" t="inlineStr">
-        <is>
-          <t>migrations/*.sql</t>
-        </is>
-      </c>
-      <c r="H3" s="12" t="inlineStr">
-        <is>
-          <t>schema_version table</t>
-        </is>
-      </c>
-      <c r="I3" s="12" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="J3" s="13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K3" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L3" s="12" t="inlineStr">
-        <is>
-          <t>scripts/db_migrate.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="12" t="inlineStr">
-        <is>
-          <t>PY-03</t>
-        </is>
-      </c>
-      <c r="B4" s="12" t="inlineStr">
-        <is>
-          <t>set_secret.py</t>
-        </is>
-      </c>
-      <c r="C4" s="12" t="inlineStr">
-        <is>
-          <t>Store a secret value from a hidden prompt or file (never a CLI arg); verify KMS key; never echo</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E4" s="12" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="F4" s="12" t="inlineStr">
-        <is>
-          <t>secretsmanager, kms</t>
-        </is>
-      </c>
-      <c r="G4" s="12" t="inlineStr">
-        <is>
-          <t>secret name</t>
-        </is>
-      </c>
-      <c r="H4" s="12" t="inlineStr">
-        <is>
-          <t>secret version id</t>
-        </is>
-      </c>
-      <c r="I4" s="12" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="J4" s="13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K4" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L4" s="12" t="inlineStr">
-        <is>
-          <t>scripts/set_secret.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="12" t="inlineStr">
-        <is>
-          <t>PY-04</t>
-        </is>
-      </c>
-      <c r="B5" s="12" t="inlineStr">
-        <is>
-          <t>bedrock_smoke_test.py</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>Confirm India-profile model access, latency and token cost for a test prompt</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E5" s="12" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="F5" s="12" t="inlineStr">
-        <is>
-          <t>bedrock:InvokeModel</t>
-        </is>
-      </c>
-      <c r="G5" s="12" t="inlineStr">
-        <is>
-          <t>model ids</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>latency / cost report</t>
-        </is>
-      </c>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="J5" s="13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K5" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L5" s="12" t="inlineStr">
-        <is>
-          <t>scripts/bedrock_smoke_test.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="12" t="inlineStr">
-        <is>
-          <t>PY-05</t>
-        </is>
-      </c>
-      <c r="B6" s="12" t="inlineStr">
-        <is>
-          <t>aurora_wake_check.py</t>
-        </is>
-      </c>
-      <c r="C6" s="12" t="inlineStr">
-        <is>
-          <t>Measure Aurora resume time after auto-pause; tune retry/backoff</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E6" s="12" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="F6" s="12" t="inlineStr">
-        <is>
-          <t>rds-data</t>
-        </is>
-      </c>
-      <c r="G6" s="12" t="inlineStr">
-        <is>
-          <t>cluster ARN</t>
-        </is>
-      </c>
-      <c r="H6" s="12" t="inlineStr">
-        <is>
-          <t>resume seconds</t>
-        </is>
-      </c>
-      <c r="I6" s="12" t="inlineStr">
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>&lt;1 GB test data</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="F8" s="12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G8" s="12">
+        <f>F8*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>$0.11/GB-mo + $0.22/M I/O (verified rates); volume estimate</t>
+        </is>
+      </c>
+      <c r="I8" s="12" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
+        <is>
+          <t>Lambda ×2 + Function URL</t>
+        </is>
+      </c>
+      <c r="C9" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-dev-api / weekend2-dev-worker</t>
+        </is>
+      </c>
+      <c r="D9" s="12" t="inlineStr">
+        <is>
+          <t>python3.14 arm64; AWS_IAM URL; BUFFERED</t>
+        </is>
+      </c>
+      <c r="E9" s="12" t="inlineStr">
+        <is>
+          <t>Always free: 1M req + 400k GB-s/mo</t>
+        </is>
+      </c>
+      <c r="F9" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="12">
+        <f>F9*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H9" s="12" t="inlineStr">
+        <is>
+          <t>AWS Free Tier (always free)</t>
+        </is>
+      </c>
+      <c r="I9" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="J9" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>CloudWatch Logs ×2</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="inlineStr">
+        <is>
+          <t>/aws/lambda/weekend2-dev-*</t>
+        </is>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>3-day retention; KMS; DEBUG</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>5 GB ingest free (Not verified)</t>
+        </is>
+      </c>
+      <c r="F10" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G10" s="12">
+        <f>F10*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H10" s="12" t="inlineStr">
+        <is>
+          <t>$0.67/GB ingest; volume estimate</t>
+        </is>
+      </c>
+      <c r="I10" s="12" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>EventBridge Scheduler</t>
+        </is>
+      </c>
+      <c r="C11" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-dev group + 2 daily jobs</t>
+        </is>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>IST cron</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>14M invocations/mo free (Not verified)</t>
+        </is>
+      </c>
+      <c r="F11" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="12">
+        <f>F11*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H11" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="J6" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K6" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L6" s="12" t="inlineStr">
-        <is>
-          <t>scripts/aurora_wake_check.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="12" t="inlineStr">
-        <is>
-          <t>PY-06</t>
-        </is>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
-        <is>
-          <t>secret_scan.py</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>Pre-commit/CI guard for the public repo: gitleaks + regex for account IDs, IPs, keys</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="E7" s="12" t="inlineStr">
-        <is>
-          <t>pre-commit / CI</t>
-        </is>
-      </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="I11" s="12" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="J11" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="12" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="12" t="inlineStr">
+        <is>
+          <t>EC2 t4g.small (entry node)</t>
+        </is>
+      </c>
+      <c r="C12" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-dev-entry (tailnet node-d1)</t>
+        </is>
+      </c>
+      <c r="D12" s="12" t="inlineStr">
+        <is>
+          <t>AL2023 arm64; IMDSv2; SSM; tag:weekend-dev; can be disabled</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="inlineStr">
+        <is>
+          <t>EC2 T4g free trial: 750 h/mo, ap-south-1, until 2026-12-31</t>
+        </is>
+      </c>
+      <c r="F12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="12">
+        <f>F12*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H12" s="12" t="inlineStr">
+        <is>
+          <t>aws.amazon.com/ec2/faqs (read 2026-10-02)</t>
+        </is>
+      </c>
+      <c r="I12" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="J12" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>EBS gp3 8 GB</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>(root volume)</t>
+        </is>
+      </c>
+      <c r="D13" s="12" t="inlineStr">
+        <is>
+          <t>Encrypted with CMK; billed even when the node is stopped</t>
+        </is>
+      </c>
+      <c r="E13" s="12" t="inlineStr">
+        <is>
+          <t>Not covered by T4g trial</t>
+        </is>
+      </c>
+      <c r="F13" s="12">
+        <f>IF($F$27&gt;0,ROUND(0.0912*8,2),0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="12">
+        <f>F13*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>$0.0912/GB-mo × 8 (2026-09-25)</t>
+        </is>
+      </c>
+      <c r="I13" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="J13" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>Public IPv4</t>
+        </is>
+      </c>
+      <c r="C14" s="12" t="inlineStr">
+        <is>
+          <t>(auto-assigned)</t>
+        </is>
+      </c>
+      <c r="D14" s="12" t="inlineStr">
+        <is>
+          <t>Egress only; released while the node is stopped</t>
+        </is>
+      </c>
+      <c r="E14" s="12" t="inlineStr">
+        <is>
+          <t>No free tier listed on VPC pricing page</t>
+        </is>
+      </c>
+      <c r="F14" s="12">
+        <f>ROUND(0.005*$F$27,2)</f>
+        <v/>
+      </c>
+      <c r="G14" s="12">
+        <f>F14*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>$0.005/h × running hours (F27); aws.amazon.com/vpc/pricing</t>
+        </is>
+      </c>
+      <c r="I14" s="12" t="inlineStr">
+        <is>
+          <t>Verified</t>
+        </is>
+      </c>
+      <c r="J14" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>S3 backup bucket</t>
+        </is>
+      </c>
+      <c r="C15" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-dev-backups-&lt;account-id&gt;</t>
+        </is>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Object Lock 1 day; force_destroy; SSE-KMS</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="G7" s="12" t="inlineStr">
-        <is>
-          <t>staged files</t>
-        </is>
-      </c>
-      <c r="H7" s="12" t="inlineStr">
-        <is>
-          <t>pass / fail</t>
-        </is>
-      </c>
-      <c r="I7" s="12" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="J7" s="13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K7" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L7" s="12" t="inlineStr">
-        <is>
-          <t>scripts/secret_scan.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="12" t="inlineStr">
-        <is>
-          <t>PY-07</t>
-        </is>
-      </c>
-      <c r="B8" s="12" t="inlineStr">
-        <is>
-          <t>bootstrap_owner.py</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="inlineStr">
-        <is>
-          <t>Create the single owner row + one-time passkey registration code (shown once over SSM)</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E8" s="12" t="inlineStr">
-        <is>
-          <t>Manual, once</t>
-        </is>
-      </c>
-      <c r="F8" s="12" t="inlineStr">
-        <is>
-          <t>rds-data, secretsmanager</t>
-        </is>
-      </c>
-      <c r="G8" s="12" t="inlineStr">
+      <c r="F15" s="12" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="G15" s="12">
+        <f>F15*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Test-sized</t>
+        </is>
+      </c>
+      <c r="I15" s="12" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="J15" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>AWS Budget</t>
+        </is>
+      </c>
+      <c r="C16" s="12" t="inlineStr">
+        <is>
+          <t>weekend2-dev-monthly</t>
+        </is>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>USD 12 incl. tax; 50/80/100% + forecast</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Budgets free (no actions)</t>
+        </is>
+      </c>
+      <c r="F16" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="12">
+        <f>F16*Cost!$B$15</f>
+        <v/>
+      </c>
+      <c r="H16" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H8" s="12" t="inlineStr">
-        <is>
-          <t>registration code</t>
-        </is>
-      </c>
-      <c r="I8" s="12" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="J8" s="13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K8" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L8" s="12" t="inlineStr">
-        <is>
-          <t>scripts/bootstrap_owner.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
-        <is>
-          <t>PY-08</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>reminder_scheduler.py (app module)</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>Create/delete one-time EventBridge schedules for reminders (no polling)</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="inlineStr">
-        <is>
-          <t>Called by API</t>
-        </is>
-      </c>
-      <c r="F9" s="12" t="inlineStr">
-        <is>
-          <t>scheduler, iam:PassRole</t>
-        </is>
-      </c>
-      <c r="G9" s="12" t="inlineStr">
-        <is>
-          <t>reminder</t>
-        </is>
-      </c>
-      <c r="H9" s="12" t="inlineStr">
-        <is>
-          <t>schedule ARN</t>
-        </is>
-      </c>
-      <c r="I9" s="12" t="inlineStr">
-        <is>
-          <t>P5</t>
-        </is>
-      </c>
-      <c r="J9" s="13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K9" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L9" s="12" t="inlineStr">
-        <is>
-          <t>src/weekend/reminders.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="12" t="inlineStr">
-        <is>
-          <t>PY-09</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>tailscale_authkey_rotate.py</t>
-        </is>
-      </c>
-      <c r="C10" s="12" t="inlineStr">
-        <is>
-          <t>Create a new tagged Tailscale auth key via API and store it in Secrets Manager before expiry</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F10" s="12" t="inlineStr">
-        <is>
-          <t>Tailscale API, secretsmanager</t>
-        </is>
-      </c>
-      <c r="G10" s="12" t="inlineStr">
+      <c r="I16" s="12" t="inlineStr">
+        <is>
+          <t>Not verified</t>
+        </is>
+      </c>
+      <c r="J16" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Amazon Bedrock (Haiku 4.5, dev testing)</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="H10" s="12" t="inlineStr">
-        <is>
-          <t>new secret version</t>
-        </is>
-      </c>
-      <c r="I10" s="12" t="inlineStr">
-        <is>
-          <t>P4</t>
-        </is>
-      </c>
-      <c r="J10" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K10" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L10" s="12" t="inlineStr">
-        <is>
-          <t>scripts/tailscale_authkey_rotate.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="12" t="inlineStr">
-        <is>
-          <t>PY-10</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>voice_benchmark.py</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>Benchmark STT/TTS options (on-device, Transcribe, Polly, local) for latency and ₹/minute</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="F11" s="12" t="inlineStr">
-        <is>
-          <t>transcribe, polly</t>
-        </is>
-      </c>
-      <c r="G11" s="12" t="inlineStr">
-        <is>
-          <t>sample audio</t>
-        </is>
-      </c>
-      <c r="H11" s="12" t="inlineStr">
-        <is>
-          <t>benchmark table</t>
-        </is>
-      </c>
-      <c r="I11" s="12" t="inlineStr">
-        <is>
-          <t>P7</t>
-        </is>
-      </c>
-      <c r="J11" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K11" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L11" s="12" t="inlineStr">
-        <is>
-          <t>scripts/voice_benchmark.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="12" t="inlineStr">
-        <is>
-          <t>PY-11</t>
-        </is>
-      </c>
-      <c r="B12" s="12" t="inlineStr">
-        <is>
-          <t>data_export.py</t>
-        </is>
-      </c>
-      <c r="C12" s="12" t="inlineStr">
-        <is>
-          <t>Export all owner data to an encrypted archive in S3</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>Worker 03:30 IST + on demand</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="inlineStr">
-        <is>
-          <t>rds-data, s3, kms</t>
-        </is>
-      </c>
-      <c r="G12" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H12" s="12" t="inlineStr">
-        <is>
-          <t>s3://…/daily/</t>
-        </is>
-      </c>
-      <c r="I12" s="12" t="inlineStr">
-        <is>
-          <t>P6, P10</t>
-        </is>
-      </c>
-      <c r="J12" s="13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K12" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L12" s="12" t="inlineStr">
-        <is>
-          <t>scripts/data_export.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="12" t="inlineStr">
-        <is>
-          <t>PY-12</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>retention_cleanup.py</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>Delete data past its retention per table; write audit entries</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E13" s="12" t="inlineStr">
-        <is>
-          <t>Worker 03:00 IST</t>
-        </is>
-      </c>
-      <c r="F13" s="12" t="inlineStr">
-        <is>
-          <t>rds-data</t>
-        </is>
-      </c>
-      <c r="G13" s="12" t="inlineStr">
-        <is>
-          <t>retention table</t>
-        </is>
-      </c>
-      <c r="H13" s="12" t="inlineStr">
-        <is>
-          <t>deleted counts</t>
-        </is>
-      </c>
-      <c r="I13" s="12" t="inlineStr">
-        <is>
-          <t>P5, P8</t>
-        </is>
-      </c>
-      <c r="J13" s="13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K13" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L13" s="12" t="inlineStr">
-        <is>
-          <t>scripts/retention_cleanup.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>PY-13</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="inlineStr">
-        <is>
-          <t>delete_all_data.py</t>
-        </is>
-      </c>
-      <c r="C14" s="12" t="inlineStr">
-        <is>
-          <t>'Forget everything': purge DB rows + S3 objects (respecting Object Lock) with double confirmation</t>
-        </is>
-      </c>
-      <c r="D14" s="12" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="E14" s="12" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="F14" s="12" t="inlineStr">
-        <is>
-          <t>rds-data, s3</t>
-        </is>
-      </c>
-      <c r="G14" s="12" t="inlineStr">
-        <is>
-          <t>confirmation phrase</t>
-        </is>
-      </c>
-      <c r="H14" s="12" t="inlineStr">
-        <is>
-          <t>purge report</t>
-        </is>
-      </c>
-      <c r="I14" s="12" t="inlineStr">
-        <is>
-          <t>P6</t>
-        </is>
-      </c>
-      <c r="J14" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K14" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L14" s="12" t="inlineStr">
-        <is>
-          <t>scripts/delete_all_data.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="12" t="inlineStr">
-        <is>
-          <t>PY-14</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>audit_verify.py</t>
-        </is>
-      </c>
-      <c r="C15" s="12" t="inlineStr">
-        <is>
-          <t>Verify the audit_log hash chain against S3 Object Lock copies</t>
-        </is>
-      </c>
-      <c r="D15" s="12" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E15" s="12" t="inlineStr">
-        <is>
-          <t>Weekly / manual</t>
-        </is>
-      </c>
-      <c r="F15" s="12" t="inlineStr">
-        <is>
-          <t>rds-data, s3</t>
-        </is>
-      </c>
-      <c r="G15" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H15" s="12" t="inlineStr">
-        <is>
-          <t>pass / fail</t>
-        </is>
-      </c>
-      <c r="I15" s="12" t="inlineStr">
-        <is>
-          <t>P8</t>
-        </is>
-      </c>
-      <c r="J15" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K15" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L15" s="12" t="inlineStr">
-        <is>
-          <t>scripts/audit_verify.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="12" t="inlineStr">
-        <is>
-          <t>PY-15</t>
-        </is>
-      </c>
-      <c r="B16" s="12" t="inlineStr">
-        <is>
-          <t>tailnet_check.py</t>
-        </is>
-      </c>
-      <c r="C16" s="12" t="inlineStr">
-        <is>
-          <t>Check Tailscale devices/ACLs: only owner devices + tag:weekend; alert on a new device</t>
-        </is>
-      </c>
-      <c r="D16" s="12" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="E16" s="12" t="inlineStr">
-        <is>
-          <t>Daily</t>
-        </is>
-      </c>
-      <c r="F16" s="12" t="inlineStr">
-        <is>
-          <t>Tailscale API</t>
-        </is>
-      </c>
-      <c r="G16" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H16" s="12" t="inlineStr">
-        <is>
-          <t>report</t>
-        </is>
-      </c>
-      <c r="I16" s="12" t="inlineStr">
-        <is>
-          <t>P1, P9</t>
-        </is>
-      </c>
-      <c r="J16" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K16" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L16" s="12" t="inlineStr">
-        <is>
-          <t>scripts/tailnet_check.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>PY-16</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>restore_drill.py</t>
-        </is>
-      </c>
-      <c r="C17" s="12" t="inlineStr">
-        <is>
-          <t>Restore latest snapshot to a temporary cluster, run integrity checks, record result, delete the temp cluster</t>
-        </is>
-      </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>in.* India profile; both model slots = Haiku</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>Quarterly</t>
-        </is>
-      </c>
-      <c r="F17" s="12" t="inlineStr">
-        <is>
-          <t>rds, rds-data</t>
-        </is>
-      </c>
-      <c r="G17" s="12" t="inlineStr">
-        <is>
-          <t>snapshot id</t>
-        </is>
+          <t>No free tier (credits apply)</t>
+        </is>
+      </c>
+      <c r="F17" s="12">
+        <f>$F$28</f>
+        <v/>
+      </c>
+      <c r="G17" s="12">
+        <f>F17*Cost!$B$15</f>
+        <v/>
       </c>
       <c r="H17" s="12" t="inlineStr">
         <is>
-          <t>drill record</t>
+          <t>Estimate (F28)</t>
         </is>
       </c>
       <c r="I17" s="12" t="inlineStr">
         <is>
-          <t>P10</t>
-        </is>
-      </c>
-      <c r="J17" s="13" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="K17" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L17" s="12" t="inlineStr">
-        <is>
-          <t>scripts/restore_drill.py</t>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="J17" s="12" t="inlineStr">
+        <is>
+          <t>Drafted (not applied)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="12" t="inlineStr">
         <is>
-          <t>PY-17</t>
+          <t>GST</t>
         </is>
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>healthcheck.py</t>
+          <t>GST (IGST 18%)</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
         <is>
-          <t>Synthetic check via the tailnet: login page, API health, Bedrock call (runs daily, not per-minute, so Aurora can pause)</t>
+          <t>AWS India (AISPL) invoice</t>
         </is>
       </c>
       <c r="D18" s="12" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>18% of lines above; assumes AISPL billing</t>
         </is>
       </c>
       <c r="E18" s="12" t="inlineStr">
         <is>
-          <t>Daily 09:00 IST / manual</t>
-        </is>
-      </c>
-      <c r="F18" s="12" t="inlineStr">
-        <is>
-          <t>None (tailnet)</t>
-        </is>
-      </c>
-      <c r="G18" s="12" t="inlineStr">
-        <is>
           <t>—</t>
         </is>
       </c>
+      <c r="F18" s="12">
+        <f>ROUND(SUM(F2:F17)*0.18,2)</f>
+        <v/>
+      </c>
+      <c r="G18" s="12">
+        <f>F18*Cost!$B$15</f>
+        <v/>
+      </c>
       <c r="H18" s="12" t="inlineStr">
         <is>
-          <t>status report</t>
+          <t>AISPL charges 18% GST</t>
         </is>
       </c>
       <c r="I18" s="12" t="inlineStr">
         <is>
-          <t>P9</t>
-        </is>
-      </c>
-      <c r="J18" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K18" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L18" s="12" t="inlineStr">
-        <is>
-          <t>scripts/healthcheck.py</t>
+          <t>Assumption</t>
+        </is>
+      </c>
+      <c r="J18" s="12" t="inlineStr">
+        <is>
+          <t>Applies on apply</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>PY-18</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>cost_report.py</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="inlineStr">
-        <is>
-          <t>Month-to-date + forecast cost vs ₹5,000 using live FX; append to tracker</t>
-        </is>
-      </c>
-      <c r="D19" s="12" t="inlineStr">
-        <is>
-          <t>6</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>Daily / manual</t>
-        </is>
-      </c>
-      <c r="F19" s="12" t="inlineStr">
-        <is>
-          <t>ce:GetCostAndUsage, ce:GetCostForecast</t>
-        </is>
-      </c>
-      <c r="G19" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H19" s="12" t="inlineStr">
-        <is>
-          <t>INR report</t>
-        </is>
-      </c>
-      <c r="I19" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J19" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K19" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L19" s="12" t="inlineStr">
-        <is>
-          <t>scripts/cost_report.py</t>
-        </is>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Dev total per month incl. GST</t>
+        </is>
+      </c>
+      <c r="F19" s="3">
+        <f>SUM(F2:F18)</f>
+        <v/>
+      </c>
+      <c r="G19" s="3">
+        <f>SUM(G2:G18)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>PY-19</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>price_check.py</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="inlineStr">
-        <is>
-          <t>Pull AWS Price List (ap-south-1) for every tracked resource; flag changes; update Resources sheet</t>
-        </is>
-      </c>
-      <c r="D20" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>Monthly</t>
-        </is>
-      </c>
-      <c r="F20" s="12" t="inlineStr">
-        <is>
-          <t>None (public price list)</t>
-        </is>
-      </c>
-      <c r="G20" s="12" t="inlineStr">
-        <is>
-          <t>Resources sheet</t>
-        </is>
-      </c>
-      <c r="H20" s="12" t="inlineStr">
-        <is>
-          <t>updated prices</t>
-        </is>
-      </c>
-      <c r="I20" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J20" s="13" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="K20" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L20" s="12" t="inlineStr">
-        <is>
-          <t>scripts/price_check.py</t>
-        </is>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Dev budget (USD 12)</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="G20" s="3">
+        <f>F20*Cost!$B$15</f>
+        <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>PY-20</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>fx_rate_update.py</t>
-        </is>
-      </c>
-      <c r="C21" s="12" t="inlineStr">
-        <is>
-          <t>Fetch USD/INR from 3 sources, take the median, update Cost!B15 with date and sources</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E21" s="12" t="inlineStr">
-        <is>
-          <t>Daily / manual</t>
-        </is>
-      </c>
-      <c r="F21" s="12" t="inlineStr">
-        <is>
-          <t>None (public APIs)</t>
-        </is>
-      </c>
-      <c r="G21" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H21" s="12" t="inlineStr">
-        <is>
-          <t>rate + sources</t>
-        </is>
-      </c>
-      <c r="I21" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J21" s="13" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="K21" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L21" s="12" t="inlineStr">
-        <is>
-          <t>scripts/fx_rate_update.py</t>
-        </is>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Dev fits its budget?</t>
+        </is>
+      </c>
+      <c r="G21" s="3">
+        <f>IF(F19&lt;=F20,"Yes","No")</f>
+        <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>PY-21</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>tracker_sync.py</t>
-        </is>
-      </c>
-      <c r="C22" s="12" t="inlineStr">
-        <is>
-          <t>Sync tracker tables (tasks, issues, decisions) with PROJECT_MEMORY.md</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>Manual</t>
-        </is>
-      </c>
-      <c r="F22" s="12" t="inlineStr">
-        <is>
-          <t>None</t>
-        </is>
-      </c>
-      <c r="G22" s="12" t="inlineStr">
-        <is>
-          <t>tracker + memory</t>
-        </is>
-      </c>
-      <c r="H22" s="12" t="inlineStr">
-        <is>
-          <t>diff report</t>
-        </is>
-      </c>
-      <c r="I22" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J22" s="13" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="K22" s="13" t="inlineStr">
-        <is>
-          <t>Planned</t>
-        </is>
-      </c>
-      <c r="L22" s="12" t="inlineStr">
-        <is>
-          <t>scripts/tracker_sync.py</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="23" t="inlineStr">
-        <is>
-          <t>Standards: Python 3.12+ (Lambda runtime python3.14), type hints, logging (not print), argparse, explicit non-zero exits, pytest tests, ruff/black. Secrets only from Secrets Manager.</t>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Dev + prod together (₹)</t>
+        </is>
+      </c>
+      <c r="G22" s="3">
+        <f>G19+Resources!J42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Dev + prod within ₹5,000?</t>
+        </is>
+      </c>
+      <c r="G23" s="3">
+        <f>IF(G22&lt;=Cost!B16,"Yes","No — destroy dev before prod goes live")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Assumptions (yellow = edit me)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Aurora active hours / month</t>
+        </is>
+      </c>
+      <c r="F26" s="35" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>Entry node running hours / month (730 = 24/7; 0 = disabled)</t>
+        </is>
+      </c>
+      <c r="F27" s="35" t="n">
+        <v>730</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>Bedrock dev usage (USD / month)</t>
+        </is>
+      </c>
+      <c r="F28" s="35" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="36" t="inlineStr">
+        <is>
+          <t>Dev = infra/envs/dev (PROVISIONAL — depends on D1). Free tier used where it exists in ap-south-1: Lambda always free; Scheduler, Budgets and S3 cost nothing or cents at dev volume; EC2 T4g trial (t4g.small, 750 h/month, until 2026-12-31 — switch to t4g.nano before then). Not free: KMS, Secrets Manager, Aurora, public IPv4, EBS, Bedrock. A new-account sign-up credit (USD 100–200, Free plan 6 months) would cover dev. GCP not used: its always-free e2-micro exists only in US regions (data residency, P7) and D4 is AWS-provisional. Sources: aws.amazon.com/ec2/faqs, aws.amazon.com/vpc/pricing, docs.aws.amazon.com free-tier-plans (read 2026-10-02).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L22"/>
-  <conditionalFormatting sqref="K2:K200">
-    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
-      <formula>"Done"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
-      <formula>"In progress"</formula>
-    </cfRule>
-    <cfRule type="cellIs" priority="3" operator="equal" dxfId="3">
-      <formula>"Planned"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <dataValidations count="2">
-    <dataValidation sqref="K2:K200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Planned,In progress,Done,Dropped"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J2:J200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"High,Medium,Low"</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(dev): normal prod-like sizing for on-demand dev; add masked plan report script
- envs/dev: entry node t4g.nano on demand (was t4g.small free trial), Aurora 0-2 ACU,
  Haiku + Sonnet model slots - same as prod; destroy-friendly settings kept
- infra/scripts/plan_env.py: terraform plan -> ~/.tfplans + masked Markdown report
  (account ID, e-mails) for PRs; --local-state previews before bootstrap; never applies
- README: dev table, on-demand cost (~INR 682/month at 60 node-hours), plan step
- tracker v1.5: Dev env sheet re-costed; I-14 closed

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/Weekend2.0_Tracker.xlsx
+++ b/tracking/Weekend2.0_Tracker.xlsx
@@ -37,7 +37,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="₹#,##0;(₹#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -45,6 +45,7 @@
     <numFmt numFmtId="168" formatCode="$#,##0.00"/>
     <numFmt numFmtId="169" formatCode="₹#,##0"/>
     <numFmt numFmtId="170" formatCode="$#,##0.000;($#,##0.000);&quot;-&quot;"/>
+    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -2255,7 +2256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2489,6 +2490,31 @@
       <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Dev env sheet (envs/dev, free-tier sizing, ≈ ₹1,042/month incl. GST); tasks T-020, T-021; issues I-13–I-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>46297</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>Dev env: normal sizing like prod (t4g.nano on demand, Aurora 0–2 ACU, Haiku + Sonnet); node 60 h/month ≈ ₹682 incl. GST; I-14 closed</t>
         </is>
       </c>
     </row>
@@ -5016,7 +5042,7 @@
       </c>
       <c r="B15" s="12" t="inlineStr">
         <is>
-          <t>EC2 T4g free trial (t4g.small) ends 2026-12-31; dev node then becomes paid</t>
+          <t>EC2 T4g free trial (t4g.small) ends 2026-12-31 — no longer relevant: dev now uses normal t4g.nano</t>
         </is>
       </c>
       <c r="C15" s="12" t="inlineStr">
@@ -5031,13 +5057,15 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F15" s="16" t="n">
         <v>46297</v>
       </c>
-      <c r="G15" s="16" t="n"/>
+      <c r="G15" s="16" t="n">
+        <v>46297</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -8685,7 +8713,7 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>0–1 ACU; pause after 300 s; Data API; no deletion protection; 1-day backups</t>
+          <t>0–2 ACU (same as prod); pause after 300 s; Data API; no deletion protection; 1-day backups</t>
         </is>
       </c>
       <c r="E7" s="12" t="n"/>
@@ -8907,7 +8935,7 @@
       </c>
       <c r="B12" s="12" t="inlineStr">
         <is>
-          <t>EC2 t4g.small (entry node)</t>
+          <t>EC2 t4g.nano (entry node)</t>
         </is>
       </c>
       <c r="C12" s="12" t="inlineStr">
@@ -8917,16 +8945,17 @@
       </c>
       <c r="D12" s="12" t="inlineStr">
         <is>
-          <t>AL2023 arm64; IMDSv2; SSM; tag:weekend-dev; can be disabled</t>
+          <t>AL2023 arm64; IMDSv2; SSM; tag:weekend-dev; normal on-demand; stop between sessions</t>
         </is>
       </c>
       <c r="E12" s="12" t="inlineStr">
         <is>
-          <t>EC2 T4g free trial: 750 h/mo, ap-south-1, until 2026-12-31</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>0</v>
+          <t>None (normal on-demand)</t>
+        </is>
+      </c>
+      <c r="F12" s="12">
+        <f>ROUND(0.0028*$F$27,2)</f>
+        <v/>
       </c>
       <c r="G12" s="12">
         <f>F12*Cost!$B$15</f>
@@ -8934,7 +8963,7 @@
       </c>
       <c r="H12" s="12" t="inlineStr">
         <is>
-          <t>aws.amazon.com/ec2/faqs (read 2026-10-02)</t>
+          <t>$0.0028/h × running hours (F27) (AWS Price List API ap-south-1 2026-09-25)</t>
         </is>
       </c>
       <c r="I12" s="12" t="inlineStr">
@@ -9144,7 +9173,7 @@
       </c>
       <c r="B17" s="12" t="inlineStr">
         <is>
-          <t>Amazon Bedrock (Haiku 4.5, dev testing)</t>
+          <t>Amazon Bedrock (Haiku 4.5 + Sonnet, dev testing)</t>
         </is>
       </c>
       <c r="C17" s="12" t="inlineStr">
@@ -9154,7 +9183,7 @@
       </c>
       <c r="D17" s="12" t="inlineStr">
         <is>
-          <t>in.* India profile; both model slots = Haiku</t>
+          <t>in.* India profiles; same model slots as prod</t>
         </is>
       </c>
       <c r="E17" s="12" t="inlineStr">
@@ -9318,11 +9347,11 @@
     <row r="27">
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>Entry node running hours / month (730 = 24/7; 0 = disabled)</t>
+          <t>Entry node running hours / month (60 = on demand; 730 = 24/7; 0 = disabled)</t>
         </is>
       </c>
       <c r="F27" s="35" t="n">
-        <v>730</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28">
@@ -9338,7 +9367,7 @@
     <row r="30">
       <c r="A30" s="36" t="inlineStr">
         <is>
-          <t>Dev = infra/envs/dev (PROVISIONAL — depends on D1). Free tier used where it exists in ap-south-1: Lambda always free; Scheduler, Budgets and S3 cost nothing or cents at dev volume; EC2 T4g trial (t4g.small, 750 h/month, until 2026-12-31 — switch to t4g.nano before then). Not free: KMS, Secrets Manager, Aurora, public IPv4, EBS, Bedrock. A new-account sign-up credit (USD 100–200, Free plan 6 months) would cover dev. GCP not used: its always-free e2-micro exists only in US regions (data residency, P7) and D4 is AWS-provisional. Sources: aws.amazon.com/ec2/faqs, aws.amazon.com/vpc/pricing, docs.aws.amazon.com free-tier-plans (read 2026-10-02).</t>
+          <t>Dev = infra/envs/dev (PROVISIONAL — depends on D1). Normal (non-free-tier) resources sized like prod; dev runs only when needed: stop the node between sessions, destroy when idle. Always charged while deployed: KMS, Secrets Manager, EBS. Lambda is always free at this volume; Scheduler, Budgets and S3 cost nothing or cents. GCP not used: its always-free VM exists only in US regions (data residency, P7) and D4 is AWS-provisional. Sources: AWS Price List API ap-south-1 (2026-09), aws.amazon.com/vpc/pricing (read 2026-10-02).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(branching): main = base code, env values on env branches, feature_* from dev
- docs/BRANCHING.md: branch roles, values files, flow (feature -> dev, promote -> main, sync down)
- .github/workflows/branch-guard.yml: block env values on main / wrong env, secrets check,
  terraform fmt + validate (no AWS credentials; actions pinned by SHA)
- .gitignore: allow infra/envs/*/values.auto.tfvars (committed on env branches only)
- dev terraform.tfvars.example: sensitive values only
- README + tracker v1.5 (T-022, T-023, I-16)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/Weekend2.0_Tracker.xlsx
+++ b/tracking/Weekend2.0_Tracker.xlsx
@@ -37,7 +37,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="7">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="₹#,##0;(₹#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -45,6 +45,7 @@
     <numFmt numFmtId="168" formatCode="$#,##0.00"/>
     <numFmt numFmtId="169" formatCode="₹#,##0"/>
     <numFmt numFmtId="170" formatCode="$#,##0.000;($#,##0.000);&quot;-&quot;"/>
+    <numFmt numFmtId="171" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -2255,7 +2256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2489,6 +2490,31 @@
       <c r="E9" s="12" t="inlineStr">
         <is>
           <t>Dev env sheet (envs/dev, free-tier sizing, ≈ ₹1,042/month incl. GST); tasks T-020, T-021; issues I-13–I-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="12" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
+      <c r="C10" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="D10" s="12" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E10" s="12" t="inlineStr">
+        <is>
+          <t>Branching strategy (main / dev / feature_infra); T-022, T-023; I-16. Dev env sheet stays free-tier (dev branch values)</t>
         </is>
       </c>
     </row>
@@ -3496,7 +3522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I22"/>
+  <dimension ref="A1:I24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4261,6 +4287,78 @@
       <c r="I22" s="12" t="inlineStr">
         <is>
           <t>Before the dev entry node first boots</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>T-022</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" s="12" t="inlineStr">
+        <is>
+          <t>Branching strategy: main = base code; dev branch = dev values (values.auto.tfvars); feature_* from dev; CI branch guard</t>
+        </is>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F23" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G23" s="16" t="n"/>
+      <c r="H23" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="I23" s="12" t="inlineStr">
+        <is>
+          <t>docs/BRANCHING.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>T-023</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>feature_infra: plan report script + CI on dev (PR feature_infra → dev)</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G24" s="16" t="n"/>
+      <c r="H24" s="16" t="n"/>
+      <c r="I24" s="12" t="inlineStr">
+        <is>
+          <t>Supersedes PR #1</t>
         </is>
       </c>
     </row>
@@ -4554,7 +4652,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5069,6 +5167,37 @@
         <v>46297</v>
       </c>
       <c r="G16" s="16" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>I-16</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>AWS credentials on the Mac are invalid (InvalidClientTokenId); blocks terraform plan</t>
+        </is>
+      </c>
+      <c r="C17" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Configure valid credentials (prefer aws configure sso); remove dead keys from ~/.aws/credentials</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F17" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G17" s="16" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G7"/>

</xml_diff>

<commit_message>
feat(infra): dev values from GitHub environment secrets; CI plan via OIDC
- docs/BRANCHING.md v1.1: main -> dev/prod/release (prod, release idle); feature_* from dev
- terraform-plan workflow: PRs into dev write terraform.tfvars from `dev` environment secrets,
  assume a read-only OIDC role, run plan_env.py, post the masked plan as a PR comment
- branch-guard: no committed tfvars anywhere; feature_* -> dev only; prod/release idle
- bootstrap/github_oidc.tf: GitHub OIDC provider + read-only plan role (dev environment only)
- .gitignore: env values never committed; tfvars example documents the secret format
- README + tracker v1.6 (T-024, I-18)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/Weekend2.0_Tracker.xlsx
+++ b/tracking/Weekend2.0_Tracker.xlsx
@@ -2256,7 +2256,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2515,6 +2515,31 @@
       <c r="E10" s="12" t="inlineStr">
         <is>
           <t>Branching strategy (main / dev / feature_infra); T-022, T-023; I-16. Dev env sheet stays free-tier (dev branch values)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="inlineStr">
+        <is>
+          <t>1.6</t>
+        </is>
+      </c>
+      <c r="C11" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="D11" s="12" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="E11" s="12" t="inlineStr">
+        <is>
+          <t>Branches main/dev/prod/release + feature_infra; dev values moved to GitHub environment secrets; T-024, I-18</t>
         </is>
       </c>
     </row>
@@ -3522,7 +3547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4301,7 +4326,7 @@
       </c>
       <c r="C23" s="12" t="inlineStr">
         <is>
-          <t>Branching strategy: main = base code; dev branch = dev values (values.auto.tfvars); feature_* from dev; CI branch guard</t>
+          <t>Branching: main base; dev/prod/release from main (prod, release idle); feature_* from dev; env values in GitHub dev environment secrets; CI guard</t>
         </is>
       </c>
       <c r="D23" s="12" t="inlineStr">
@@ -4338,7 +4363,7 @@
       </c>
       <c r="C24" s="12" t="inlineStr">
         <is>
-          <t>feature_infra: plan report script + CI on dev (PR feature_infra → dev)</t>
+          <t>feature_infra: plan script, CI plan workflow (OIDC, secrets), GitHub plan role in bootstrap — PR feature_infra → dev</t>
         </is>
       </c>
       <c r="D24" s="12" t="inlineStr">
@@ -4359,6 +4384,39 @@
       <c r="I24" s="12" t="inlineStr">
         <is>
           <t>Supersedes PR #1</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>T-024</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Set dev environment secrets AWS_ACCOUNT_ID, ALERT_EMAIL, AURORA_ENGINE_VERSION; apply bootstrap (state + OIDC role) → AWS_PLAN_ROLE_ARN</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="n"/>
+      <c r="G25" s="16" t="n"/>
+      <c r="H25" s="16" t="n"/>
+      <c r="I25" s="12" t="inlineStr">
+        <is>
+          <t>Needs valid AWS credentials (I-16) + security checkpoint</t>
         </is>
       </c>
     </row>
@@ -4652,7 +4710,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5198,6 +5256,37 @@
         <v>46298</v>
       </c>
       <c r="G17" s="16" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>I-18</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
+        <is>
+          <t>PR plan output pending: CI plan needs AWS_PLAN_ROLE_ARN (bootstrap apply) and the remaining dev secrets</t>
+        </is>
+      </c>
+      <c r="C18" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D18" s="12" t="inlineStr">
+        <is>
+          <t>T-024</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F18" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G18" s="16" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G7"/>

</xml_diff>

<commit_message>
feat(gcp): free-by-default dev (costed items on hold); fix plan bug
- Switches, default off in dev ("on hold"): enable_cmek (KMS in bootstrap/dev),
  entry_node_enabled, entry_node_egress (nat | external_ip); network NAT optional
- Free locations: state + backup buckets in US-CENTRAL1 (5 GB free); everything else
  stays inside GCP free tiers; prod keeps CMEK + NAT
- Fix: app module for_each over unknown secret IDs -> static-key map (api_secrets)
- Bootstrap reads project data only when CMEK is on, so the first plan works before
  the Cloud Resource Manager API is enabled (read-only plan: 26 to add)
- Docs: on-hold table, project weekend2-0, closed billing account; DESIGN 0.2.1;
  tracker 1.8 (I-24 billing closed, I-25 project name, T-029)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/Weekend2.0_Tracker.xlsx
+++ b/tracking/Weekend2.0_Tracker.xlsx
@@ -2193,7 +2193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2300,6 +2300,56 @@
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>Create GCP project weekend2-0 ("WeekEnd2-0"), no billing; read-only inventory of 5 existing projects</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>Google Cloud</t>
+        </is>
+      </c>
+      <c r="D5" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Delete branch archive/pr1-normal-sizing (closed PR #1, superseded AWS work)</t>
+        </is>
+      </c>
+      <c r="C6" s="12" t="inlineStr">
+        <is>
+          <t>github.com/SharoffNIKHIL/Weekend2.0</t>
+        </is>
+      </c>
+      <c r="D6" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E6" s="12" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
@@ -2322,7 +2372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2681,6 +2731,56 @@
       <c r="E14" s="12" t="inlineStr">
         <is>
           <t>Cloud switched to GCP: Resources (32 GCP lines), Cost, Dev env rebuilt; D4 decided; AWS-only issues closed; I-19–I-23; T-025–T-028; Automation Scripts on GCP services</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>DESIGN.md</t>
+        </is>
+      </c>
+      <c r="B15" s="12" t="inlineStr">
+        <is>
+          <t>0.2.1</t>
+        </is>
+      </c>
+      <c r="C15" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="D15" s="12" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="E15" s="12" t="inlineStr">
+        <is>
+          <t>Dev free by default (CMEK/entry node/NAT on hold); project weekend2-0; billing account closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="D16" s="12" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E16" s="12" t="inlineStr">
+        <is>
+          <t>Dev env free by default (≈ ₹113 = Claude usage only); T-026 progress, T-029; I-24 billing closed, I-25 project name</t>
         </is>
       </c>
     </row>
@@ -3688,7 +3788,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4355,7 +4455,7 @@
       <c r="H19" s="14" t="n"/>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>~~Aurora version + Bedrock IDs~~ superseded by D4 = GCP</t>
+          <t>Blocked: Model Garden enablement needs an open billing account (I-24)</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4709,7 @@
       </c>
       <c r="C27" s="12" t="inlineStr">
         <is>
-          <t>gcloud auth login + application-default login; create weekend2-dev-&lt;suffix&gt;, link billing</t>
+          <t>gcloud auth login ✅; create project weekend2-0 ("WeekEnd2-0") ✅ 2026-10-03; re-open billing + link ⏸; gcloud auth application-default login</t>
         </is>
       </c>
       <c r="D27" s="12" t="inlineStr">
@@ -4619,10 +4719,12 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F27" s="16" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F27" s="16" t="n">
+        <v>46298</v>
+      </c>
       <c r="G27" s="16" t="n"/>
       <c r="H27" s="16" t="n"/>
       <c r="I27" s="12" t="inlineStr">
@@ -4694,6 +4796,43 @@
       <c r="I29" s="12" t="inlineStr">
         <is>
           <t>I-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>T-029</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Free-by-default dev: CMEK / entry node / NAT behind switches (off); fix for_each bug; bootstrap read-only plan 26 to add</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G30" s="16" t="n"/>
+      <c r="H30" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="I30" s="12" t="inlineStr">
+        <is>
+          <t>feature_infra</t>
         </is>
       </c>
     </row>
@@ -4997,7 +5136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5570,7 +5709,7 @@
       </c>
       <c r="B18" s="12" t="inlineStr">
         <is>
-          <t>PR #2 plan output pending: CI plan needs GCP_WIF_PROVIDER / GCP_PLAN_SERVICE_ACCOUNT (bootstrap apply) and the dev secrets</t>
+          <t>PR #2: bootstrap plan posted (26 to add); envs/dev plan blocked until bootstrap enables project APIs (needs open billing)</t>
         </is>
       </c>
       <c r="C18" s="12" t="inlineStr">
@@ -5632,7 +5771,7 @@
       </c>
       <c r="B20" s="12" t="inlineStr">
         <is>
-          <t>gcloud tokens on the Mac expired (invalid_grant); default project is an unrelated one</t>
+          <t>gcloud user login works (2026-10-03); Application Default Credentials (used by Terraform) still expired</t>
         </is>
       </c>
       <c r="C20" s="12" t="inlineStr">
@@ -5642,7 +5781,7 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>gcloud auth login + application-default login; set a weekend2 project (T-026)</t>
+          <t>gcloud auth application-default login; set quota project weekend2-0</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -5747,6 +5886,68 @@
         <v>46298</v>
       </c>
       <c r="G23" s="16" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>I-24</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>The only billing account ("My Billing Account", INR) is CLOSED; no project has billing. Blocks every apply and Claude enablement in Model Garden</t>
+        </is>
+      </c>
+      <c r="C24" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Re-open it or create a new billing account (Console → Billing), then link weekend2-0 (checkpoint)</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F24" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G24" s="16" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>I-25</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>Project display name "WeekEnd2.0" rejected by Google (no "." allowed); created as "WeekEnd2-0", ID weekend2-0</t>
+        </is>
+      </c>
+      <c r="C25" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D25" s="12" t="inlineStr">
+        <is>
+          <t>Accept, or rename in Console (display name only)</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F25" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G25" s="16" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G7"/>
@@ -8689,7 +8890,6 @@
       <c r="I45" s="3" t="n"/>
       <c r="J45" s="3" t="n"/>
     </row>
-    <row r="46"/>
     <row r="47">
       <c r="A47" s="23" t="n"/>
     </row>
@@ -8872,7 +9072,7 @@
       </c>
       <c r="E3" s="12" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>None — ⏸ ON HOLD (only with the entry node)</t>
         </is>
       </c>
       <c r="F3" s="12">
@@ -8905,7 +9105,7 @@
       </c>
       <c r="B4" s="12" t="inlineStr">
         <is>
-          <t>KMS key (bootstrap)</t>
+          <t>KMS key (bootstrap) — ⏸ ON HOLD</t>
         </is>
       </c>
       <c r="C4" s="12" t="inlineStr">
@@ -8915,7 +9115,7 @@
       </c>
       <c r="D4" s="12" t="inlineStr">
         <is>
-          <t>CMEK, asia-south1</t>
+          <t>enable_cmek = false → Google-managed encryption</t>
         </is>
       </c>
       <c r="E4" s="12" t="inlineStr">
@@ -8924,7 +9124,7 @@
         </is>
       </c>
       <c r="F4" s="12" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="G4" s="12">
         <f>F4*Cost!$B$15</f>
@@ -8932,7 +9132,7 @@
       </c>
       <c r="H4" s="12" t="inlineStr">
         <is>
-          <t>$0.06/version + ops</t>
+          <t>$0.06/version + ops when switched on (≈ $0.10)</t>
         </is>
       </c>
       <c r="I4" s="12" t="inlineStr">
@@ -9056,16 +9256,16 @@
       </c>
       <c r="D7" s="12" t="inlineStr">
         <is>
-          <t>1-day retention; no soft delete; force_destroy</t>
+          <t>US-CENTRAL1; 1-day retention; no soft delete; force_destroy</t>
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>None (5 GB free only in US regions)</t>
+          <t>5 GB Standard free in US regions</t>
         </is>
       </c>
       <c r="F7" s="12" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="G7" s="12">
         <f>F7*Cost!$B$15</f>
@@ -9073,7 +9273,7 @@
       </c>
       <c r="H7" s="12" t="inlineStr">
         <is>
-          <t>Test-sized</t>
+          <t>Always free (US-CENTRAL1)</t>
         </is>
       </c>
       <c r="I7" s="12" t="inlineStr">
@@ -9187,7 +9387,7 @@
       </c>
       <c r="B10" s="12" t="inlineStr">
         <is>
-          <t>Compute Engine e2-micro (entry node)</t>
+          <t>Compute Engine e2-micro (entry node) — ⏸ ON HOLD</t>
         </is>
       </c>
       <c r="C10" s="12" t="inlineStr">
@@ -9299,8 +9499,9 @@
           <t>None</t>
         </is>
       </c>
-      <c r="F12" s="12" t="n">
-        <v>0.01</v>
+      <c r="F12" s="12">
+        <f>IF($F$23&gt;0,0.01,0)</f>
+        <v/>
       </c>
       <c r="G12" s="12">
         <f>F12*Cost!$B$15</f>
@@ -9566,11 +9767,11 @@
     <row r="23">
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Entry node running hours / month (730 = 24/7; 0 = disabled)</t>
+          <t>Entry node running hours / month (0 = on hold/disabled; 730 = 24/7)</t>
         </is>
       </c>
       <c r="F23" s="35" t="n">
-        <v>730</v>
+        <v>0</v>
       </c>
       <c r="G23" s="3" t="n"/>
     </row>
@@ -9590,7 +9791,7 @@
     <row r="26">
       <c r="A26" s="36" t="inlineStr">
         <is>
-          <t>Dev = infra/envs/dev on Google Cloud (D4 = GCP, 2026-10-03; D1/D2 PROVISIONAL). Free tier used wherever GCP has one: always-free e2-micro + 30 GB pd-standard in us-central1 (dev holds no real personal data; prod stays in asia-south1), Cloud Run / Firestore / Secret Manager / Scheduler / Tasks / Logging free tiers. Not free: Cloud NAT, KMS key, Vertex AI. GCP free VM regions are US-only. Sources: cloud.google.com/free, gcloud-compute.com/e2-micro.html, cloud.google.com/nat (read 2026-10-03).</t>
+          <t>Dev = infra/envs/dev, project weekend2-0 ("WeekEnd2-0", created 2026-10-03, no billing linked). FREE BY DEFAULT: costed items are switches that default to off (⏸): enable_cmek, entry_node_enabled (+ NAT egress). Free: Cloud Run, Firestore quota, Secret Manager ≤ 6 versions, Scheduler 2 of 3 jobs, Tasks, Logging, budget, GCS in US-CENTRAL1 (5 GB). Vertex AI Claude is usage-only and blocked until billing is open. Every apply needs an OPEN billing account (the current one is closed). Sources: cloud.google.com/free, cloud.google.com/nat (read 2026-10-03).</t>
         </is>
       </c>
       <c r="D26" s="5" t="n"/>
@@ -9604,7 +9805,6 @@
       <c r="D28" s="5" t="n"/>
       <c r="F28" s="42" t="n"/>
     </row>
-    <row r="29"/>
     <row r="30">
       <c r="A30" s="36" t="n"/>
     </row>

</xml_diff>

<commit_message>
feat(scripts): read-only GCP pre-flight check (gcp_check.py)
- Checks gcloud login, Application Default Credentials, billing account open/linked,
  project billing enabled and required APIs; masks billing IDs; never changes anything
- README pre-flight step; tracker 1.9 (I-24 billing still closed, I-26 console APIs, T-030)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/Weekend2.0_Tracker.xlsx
+++ b/tracking/Weekend2.0_Tracker.xlsx
@@ -2372,7 +2372,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2781,6 +2781,31 @@
       <c r="E16" s="12" t="inlineStr">
         <is>
           <t>Dev env free by default (≈ ₹113 = Claude usage only); T-026 progress, T-029; I-24 billing closed, I-25 project name</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="C17" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="D17" s="12" t="inlineStr">
+        <is>
+          <t>Patch</t>
+        </is>
+      </c>
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>Connection re-test: billing still closed (I-24), I-26 console default APIs, T-030 gcp_check.py</t>
         </is>
       </c>
     </row>
@@ -3788,7 +3813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4833,6 +4858,43 @@
       <c r="I30" s="12" t="inlineStr">
         <is>
           <t>feature_infra</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>T-030</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Read-only GCP pre-flight script infra/scripts/gcp_check.py (login, ADC, billing, APIs)</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G31" s="16" t="n"/>
+      <c r="H31" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="I31" s="12" t="inlineStr">
+        <is>
+          <t>Current result: BLOCKED (ADC expired, billing closed)</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5198,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5895,7 +5957,7 @@
       </c>
       <c r="B24" s="12" t="inlineStr">
         <is>
-          <t>The only billing account ("My Billing Account", INR) is CLOSED; no project has billing. Blocks every apply and Claude enablement in Model Garden</t>
+          <t>Billing account ("My Billing Account", INR) still reports CLOSED (re-checked 2026-10-03 after owner enabled it); weekend2-0 is linked but billingEnabled = False. Blocks applies and Claude enablement</t>
         </is>
       </c>
       <c r="C24" s="12" t="inlineStr">
@@ -5905,7 +5967,7 @@
       </c>
       <c r="D24" s="12" t="inlineStr">
         <is>
-          <t>Re-open it or create a new billing account (Console → Billing), then link weekend2-0 (checkpoint)</t>
+          <t>Check Console → Billing → account status/payment verification; re-run infra/scripts/gcp_check.py until READY</t>
         </is>
       </c>
       <c r="E24" s="12" t="inlineStr">
@@ -5948,6 +6010,37 @@
         <v>46298</v>
       </c>
       <c r="G25" s="16" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>I-26</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>Console auto-enabled ~30 default APIs on weekend2-0 (BigQuery, Gemini Cloud Assist, Dataplex, …); not used by the stack</t>
+        </is>
+      </c>
+      <c r="C26" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D26" s="12" t="inlineStr">
+        <is>
+          <t>Leave (no cost without usage) or disable unused ones later</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F26" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G26" s="16" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G7"/>

</xml_diff>

<commit_message>
chore(tracker): v2.1 — verification, D2 decided, CI/CD tasks, new issues
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tracking/Weekend2.0_Tracker.xlsx
+++ b/tracking/Weekend2.0_Tracker.xlsx
@@ -774,7 +774,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L24"/>
+  <dimension ref="A1:L27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -2155,10 +2155,197 @@
         </is>
       </c>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="A24" s="23" t="inlineStr">
         <is>
           <t>Standards: Python 3.12+ (Cloud Run container on a pinned python:3.12-slim digest), type hints, logging (not print), argparse, explicit non-zero exits, pytest tests (Firestore emulator), ruff/black. Secrets only from Secret Manager; no JSON service-account keys; GCP access through attached service accounts or Workload Identity Federation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>PY-22</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>infra/scripts/tf.py</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Local Terraform with a 1-hour impersonated token (no keys/ADC)</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>iam.serviceAccountTokenCreator on the deployer</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>values + ../credentials</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>plan/apply</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>infra/scripts/tf.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="23" t="inlineStr">
+        <is>
+          <t>PY-23</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>infra/scripts/cost_guard.py</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Block CD applies that are not free of cost</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>CI/CD</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>plan JSON</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>pass/fail</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>infra/scripts/cost_guard.py</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="23" t="inlineStr">
+        <is>
+          <t>PY-24</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>infra/scripts/promote.py</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Move code between branches; each keeps its own env values</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Manual</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>git branches</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>promote/* branch</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>P4</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>infra/scripts/promote.py</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2380,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2375,6 +2562,31 @@
         </is>
       </c>
       <c r="E7" s="12" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Install Terraform 1.16.5 (SHA256 verified), ruff, gh; merge PR #3 into dev; write CI/CD (auto-apply free resources only); deployer SA (least privilege); D2 = Vertex global; branch model option A</t>
+        </is>
+      </c>
+      <c r="C8" s="12" t="inlineStr">
+        <is>
+          <t>Mac + github.com/SharoffNIKHIL/Weekend2.0 + GCP weekend2-0</t>
+        </is>
+      </c>
+      <c r="D8" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E8" s="12" t="inlineStr">
         <is>
           <t>Owner</t>
         </is>
@@ -2397,7 +2609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2906,6 +3118,106 @@
       <c r="E20" s="12" t="inlineStr">
         <is>
           <t>Phase 1 started (Feature_code, Java); infra merged to dev; billing fixed (I-24 closed); T-031–T-036; I-27, I-28</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>DESIGN.md</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>0.4.0</t>
+        </is>
+      </c>
+      <c r="C21" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="D21" s="12" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>D2 decided (Claude on Vertex global + copy in Firestore); CI/CD; generic stack; short-lived credentials</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>ADR-0002</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="C22" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="D22" s="12" t="inlineStr">
+        <is>
+          <t>Initial</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>D2 model = Claude on Vertex AI (global)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="12" t="inlineStr">
+        <is>
+          <t>BRANCHING.md</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>1.4</t>
+        </is>
+      </c>
+      <c r="C23" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>One generic root; env values on env branches (option A); promote.py; CI/CD</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="12" t="inlineStr">
+        <is>
+          <t>Tracker</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="D24" s="12" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>Verification results, D2, CI/CD tasks T-037–T-045, issues I-29–I-35, PY-22–24</t>
         </is>
       </c>
     </row>
@@ -3678,7 +3990,7 @@
       <c r="G2" s="14" t="n"/>
       <c r="H2" s="13" t="inlineStr">
         <is>
-          <t>DESIGN.md v0.1.3; diagrams 01–05; READMEs</t>
+          <t>DESIGN.md v0.4.0; ADR-0001 (D4), ADR-0002 (D2); diagrams 01–05; READMEs</t>
         </is>
       </c>
       <c r="I2" s="15">
@@ -3716,7 +4028,7 @@
       <c r="G3" s="14" t="n"/>
       <c r="H3" s="13" t="inlineStr">
         <is>
-          <t>Feature_code: Java 17 / Spring Boot 4.1 app core in app/, 40 tests passing, local smoke test OK (PR into dev). Started early with owner approval; Phase 0 decisions D1/D2 still provisional</t>
+          <t>Java 17 / Spring Boot 4.1 app merged into dev (PR #3); 40/40 tests + 15-step smoke test 2026-10-03</t>
         </is>
       </c>
       <c r="I3" s="15">
@@ -3840,13 +4152,19 @@
       </c>
       <c r="D7" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="E7" s="14" t="n"/>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="n">
+        <v>46298</v>
+      </c>
       <c r="F7" s="14" t="n"/>
       <c r="G7" s="14" t="n"/>
-      <c r="H7" s="13" t="inlineStr"/>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>CI/CD built 2026-10-03: infra-ci/cd, app-ci/cd, branch-guard; generic infra/stack; deployer SA (code); not applied</t>
+        </is>
+      </c>
       <c r="I7" s="15">
         <f>IFERROR(COUNTIFS(Tasks!$B$2:$B$200,A7,Tasks!$E$2:$E$200,"Done")/COUNTIF(Tasks!$B$2:$B$200,A7),0)</f>
         <v/>
@@ -3919,7 +4237,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I37"/>
+  <dimension ref="A1:I46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -4219,17 +4537,19 @@
       </c>
       <c r="E8" s="13" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F8" s="14" t="n">
         <v>46297</v>
       </c>
       <c r="G8" s="14" t="n"/>
-      <c r="H8" s="14" t="n"/>
+      <c r="H8" s="14" t="n">
+        <v>46298</v>
+      </c>
       <c r="I8" s="13" t="inlineStr">
         <is>
-          <t>Diff awaiting owner approval</t>
+          <t>Memory updated 2026-10-03 (verification, D2, CI/CD, credentials)</t>
         </is>
       </c>
     </row>
@@ -4320,15 +4640,19 @@
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
-        </is>
-      </c>
-      <c r="F11" s="14" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F11" s="14" t="n">
+        <v>46298</v>
+      </c>
       <c r="G11" s="14" t="n"/>
-      <c r="H11" s="14" t="n"/>
+      <c r="H11" s="14" t="n">
+        <v>46298</v>
+      </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>Depends on D1</t>
+          <t>D2 = Claude on Vertex AI global; copy of every exchange in Firestore (ADR-0002)</t>
         </is>
       </c>
     </row>
@@ -4353,15 +4677,17 @@
       </c>
       <c r="E12" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F12" s="14" t="n"/>
       <c r="G12" s="14" t="n"/>
-      <c r="H12" s="14" t="n"/>
+      <c r="H12" s="14" t="n">
+        <v>46298</v>
+      </c>
       <c r="I12" s="13" t="inlineStr">
         <is>
-          <t>Depends on D1, D2</t>
+          <t>Decided 2026-10-03 (ADR-0001)</t>
         </is>
       </c>
     </row>
@@ -4417,7 +4743,7 @@
       </c>
       <c r="E14" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Blocked</t>
         </is>
       </c>
       <c r="F14" s="14" t="n"/>
@@ -4425,7 +4751,7 @@
       <c r="H14" s="14" t="n"/>
       <c r="I14" s="13" t="inlineStr">
         <is>
-          <t>Then purge or archive the old repo</t>
+          <t>Owner: which service issued the v1 token? v1 repo is not on the Mac; revoke in that console (agent cannot sign in)</t>
         </is>
       </c>
     </row>
@@ -4479,13 +4805,19 @@
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F16" s="14" t="n"/>
       <c r="G16" s="14" t="n"/>
-      <c r="H16" s="14" t="n"/>
-      <c r="I16" s="13" t="inlineStr"/>
+      <c r="H16" s="14" t="n">
+        <v>46298</v>
+      </c>
+      <c r="I16" s="13" t="inlineStr">
+        <is>
+          <t>Repo exists (public, owner choice)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -4578,7 +4910,7 @@
       </c>
       <c r="E19" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
       <c r="F19" s="14" t="n"/>
@@ -4586,7 +4918,7 @@
       <c r="H19" s="14" t="n"/>
       <c r="I19" s="13" t="inlineStr">
         <is>
-          <t>Blocked: Model Garden enablement needs an open billing account (I-24)</t>
+          <t>Owner: Console → Model Garden → Claude Haiku 4.5 → Enable (free; pay per token). Billing now open</t>
         </is>
       </c>
     </row>
@@ -4611,13 +4943,19 @@
       </c>
       <c r="E20" s="13" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F20" s="14" t="n"/>
       <c r="G20" s="14" t="n"/>
-      <c r="H20" s="14" t="n"/>
-      <c r="I20" s="13" t="inlineStr"/>
+      <c r="H20" s="14" t="n">
+        <v>46298</v>
+      </c>
+      <c r="I20" s="13" t="inlineStr">
+        <is>
+          <t>Terraform 1.16.5 installed (SHA256 verified); brew 1.5.7 unlinked</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="12" t="inlineStr">
@@ -4650,7 +4988,7 @@
       <c r="H21" s="16" t="n"/>
       <c r="I21" s="12" t="inlineStr">
         <is>
-          <t>infra/README.md → Dev run order</t>
+          <t>Not deployed (owner: "don't deploy yet"). Run via infra/scripts/tf.py or infra-cd after approval</t>
         </is>
       </c>
     </row>
@@ -4790,7 +5128,7 @@
       <c r="H25" s="16" t="n"/>
       <c r="I25" s="12" t="inlineStr">
         <is>
-          <t>Needs gcloud auth login (I-20) + dev project (T-026) + security checkpoint</t>
+          <t>Now: environments dev + dev-apply secrets (infra/README.md → CI/CD); TFVARS secret retired</t>
         </is>
       </c>
     </row>
@@ -4852,17 +5190,19 @@
       </c>
       <c r="E27" s="12" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F27" s="16" t="n">
         <v>46298</v>
       </c>
       <c r="G27" s="16" t="n"/>
-      <c r="H27" s="16" t="n"/>
+      <c r="H27" s="16" t="n">
+        <v>46298</v>
+      </c>
       <c r="I27" s="12" t="inlineStr">
         <is>
-          <t>Security checkpoint (new project + billing)</t>
+          <t>Billing linked and enabled (checked 2026-10-03)</t>
         </is>
       </c>
     </row>
@@ -4920,15 +5260,17 @@
       </c>
       <c r="E29" s="12" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F29" s="16" t="n"/>
       <c r="G29" s="16" t="n"/>
-      <c r="H29" s="16" t="n"/>
+      <c r="H29" s="16" t="n">
+        <v>46298</v>
+      </c>
       <c r="I29" s="12" t="inlineStr">
         <is>
-          <t>I-19</t>
+          <t>Global accepted by owner (ADR-0002)</t>
         </is>
       </c>
     </row>
@@ -5064,17 +5406,19 @@
       </c>
       <c r="E33" s="12" t="inlineStr">
         <is>
-          <t>In progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="F33" s="16" t="n">
         <v>46298</v>
       </c>
       <c r="G33" s="16" t="n"/>
-      <c r="H33" s="16" t="n"/>
+      <c r="H33" s="16" t="n">
+        <v>46298</v>
+      </c>
       <c r="I33" s="12" t="inlineStr">
         <is>
-          <t>PR Feature_code → dev; merge after review + CI</t>
+          <t>Merged PR #3 → dev (b3dbcab). Verified 40/40 tests + 15-step smoke test</t>
         </is>
       </c>
     </row>
@@ -5207,6 +5551,319 @@
       <c r="I37" s="12" t="inlineStr">
         <is>
           <t>Replaces pasted session token in the UI</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="inlineStr">
+        <is>
+          <t>T-037</t>
+        </is>
+      </c>
+      <c r="B38" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C38" s="12" t="inlineStr">
+        <is>
+          <t>Short-lived credentials: deployer SA (bootstrap/deployer.tf), tf.py impersonation, ../credentials config; revoke ADC</t>
+        </is>
+      </c>
+      <c r="D38" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E38" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F38" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G38" s="16" t="n"/>
+      <c r="H38" s="16" t="n"/>
+      <c r="I38" s="12" t="inlineStr">
+        <is>
+          <t>Code done (feature_cicd). Owner applies bootstrap — agent IAM grants blocked by permission system</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="inlineStr">
+        <is>
+          <t>T-038</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C39" s="12" t="inlineStr">
+        <is>
+          <t>CI/CD: infra-ci (fmt, tflint, validate, plan → PR), infra-cd (apply -auto-approve, free only, owner-approved), app-ci, app-cd</t>
+        </is>
+      </c>
+      <c r="D39" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E39" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F39" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G39" s="16" t="n"/>
+      <c r="H39" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="I39" s="12" t="inlineStr">
+        <is>
+          <t>CD off until INFRA_CD_ENABLED / APP_CD_ENABLED = true</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="inlineStr">
+        <is>
+          <t>T-039</t>
+        </is>
+      </c>
+      <c r="B40" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C40" s="12" t="inlineStr">
+        <is>
+          <t>One generic infra/stack; env values on env branches (BRANCHING 1.4, option A); main/release/prod = raw code</t>
+        </is>
+      </c>
+      <c r="D40" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E40" s="12" t="inlineStr">
+        <is>
+          <t>In progress</t>
+        </is>
+      </c>
+      <c r="F40" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G40" s="16" t="n"/>
+      <c r="H40" s="16" t="n"/>
+      <c r="I40" s="12" t="inlineStr">
+        <is>
+          <t>Committed locally on feature_cicd; owner pushes branches</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>T-040</t>
+        </is>
+      </c>
+      <c r="B41" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" s="12" t="inlineStr">
+        <is>
+          <t>Copy of every LLM exchange in Firestore asia-south1 (D2 requirement)</t>
+        </is>
+      </c>
+      <c r="D41" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E41" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F41" s="16" t="n"/>
+      <c r="G41" s="16" t="n"/>
+      <c r="H41" s="16" t="n"/>
+      <c r="I41" s="12" t="inlineStr">
+        <is>
+          <t>Feature_database</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>T-041</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>Verify Google OIDC token inside the app for /jobs/* (finding F1)</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F42" s="16" t="n"/>
+      <c r="G42" s="16" t="n"/>
+      <c r="H42" s="16" t="n"/>
+      <c r="I42" s="12" t="inlineStr">
+        <is>
+          <t>Defence in depth behind Cloud Run IAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="inlineStr">
+        <is>
+          <t>T-042</t>
+        </is>
+      </c>
+      <c r="B43" s="12" t="n">
+        <v>3</v>
+      </c>
+      <c r="C43" s="12" t="inlineStr">
+        <is>
+          <t>Persist pending confirmations with expiry (finding F2)</t>
+        </is>
+      </c>
+      <c r="D43" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E43" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F43" s="16" t="n"/>
+      <c r="G43" s="16" t="n"/>
+      <c r="H43" s="16" t="n"/>
+      <c r="I43" s="12" t="inlineStr">
+        <is>
+          <t>Feature_database</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t>T-043</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C44" s="12" t="inlineStr">
+        <is>
+          <t>GitHub: gh auth login; environments dev + dev-apply (you as reviewer); secrets; branch protection</t>
+        </is>
+      </c>
+      <c r="D44" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E44" s="12" t="inlineStr">
+        <is>
+          <t>Not started</t>
+        </is>
+      </c>
+      <c r="F44" s="16" t="n"/>
+      <c r="G44" s="16" t="n"/>
+      <c r="H44" s="16" t="n"/>
+      <c r="I44" s="12" t="inlineStr">
+        <is>
+          <t>Owner (commands in infra/README.md)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="inlineStr">
+        <is>
+          <t>T-044</t>
+        </is>
+      </c>
+      <c r="B45" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C45" s="12" t="inlineStr">
+        <is>
+          <t>Install ruff 0.16.10 and gh 2.102.0 on the Mac</t>
+        </is>
+      </c>
+      <c r="D45" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E45" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F45" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G45" s="16" t="n"/>
+      <c r="H45" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="I45" s="12" t="inlineStr">
+        <is>
+          <t>Homebrew</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>T-045</t>
+        </is>
+      </c>
+      <c r="B46" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C46" s="12" t="inlineStr">
+        <is>
+          <t>Artifact Registry repo (modules/registry, keeps 2 images in dev)</t>
+        </is>
+      </c>
+      <c r="D46" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E46" s="12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G46" s="16" t="n"/>
+      <c r="H46" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="I46" s="12" t="inlineStr">
+        <is>
+          <t>Free tier 0.5 GB — asia-south1 Not verified (I-34)</t>
         </is>
       </c>
     </row>
@@ -5348,7 +6005,7 @@
       </c>
       <c r="D3" s="13" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Decided</t>
         </is>
       </c>
       <c r="E3" s="12" t="inlineStr">
@@ -5356,9 +6013,19 @@
           <t>Claude Haiku 4.5 + Sonnet 5 on Vertex AI, global endpoint (🔓 leaves India); Gemini asia-south1 = in-India option (§7)</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr"/>
-      <c r="G3" s="14" t="n"/>
-      <c r="H3" s="13" t="inlineStr"/>
+      <c r="F3" s="13" t="inlineStr">
+        <is>
+          <t>Claude on Vertex AI (global): Haiku 4.5 + Sonnet 5; copy of every exchange in Firestore asia-south1</t>
+        </is>
+      </c>
+      <c r="G3" s="14" t="n">
+        <v>46298</v>
+      </c>
+      <c r="H3" s="13" t="inlineStr">
+        <is>
+          <t>docs/adr/ADR-0002-d2-model-claude-vertex-global.md</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -5510,7 +6177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="A1:G35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5577,7 +6244,7 @@
       </c>
       <c r="D2" s="13" t="inlineStr">
         <is>
-          <t>Rotate tokens; purge or archive the old repo</t>
+          <t>Owner: tell me which service issued the v1 token, then revoke/rotate it in that console; archive the v1 repo</t>
         </is>
       </c>
       <c r="E2" s="13" t="inlineStr">
@@ -5866,18 +6533,20 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>brew install hashicorp/tap/terraform (T-019)</t>
+          <t>Done: Terraform 1.16.5 installed 2026-10-03</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F11" s="16" t="n">
         <v>46297</v>
       </c>
-      <c r="G11" s="14" t="n"/>
+      <c r="G11" s="14" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -6001,13 +6670,15 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F15" s="16" t="n">
         <v>46297</v>
       </c>
-      <c r="G15" s="16" t="n"/>
+      <c r="G15" s="16" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -6124,18 +6795,20 @@
       </c>
       <c r="D19" s="12" t="inlineStr">
         <is>
-          <t>Accept, or pick Gemini in asia-south1 under D2 (T-028)</t>
+          <t>Accepted by owner (D2, ADR-0002); copy kept in Firestore asia-south1</t>
         </is>
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Closed</t>
         </is>
       </c>
       <c r="F19" s="16" t="n">
         <v>46298</v>
       </c>
-      <c r="G19" s="16" t="n"/>
+      <c r="G19" s="16" t="n">
+        <v>46298</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="12" t="inlineStr">
@@ -6155,7 +6828,7 @@
       </c>
       <c r="D20" s="12" t="inlineStr">
         <is>
-          <t>gcloud auth application-default login; set quota project weekend2-0</t>
+          <t>ADC no longer used: gcloud auth login + tf.py (1 h impersonated token); then gcloud auth application-default revoke</t>
         </is>
       </c>
       <c r="E20" s="12" t="inlineStr">
@@ -6417,6 +7090,227 @@
         <v>46298</v>
       </c>
       <c r="G28" s="16" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>I-29</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>/jobs/* has no in-app auth; relies on Cloud Run IAM only (F1)</t>
+        </is>
+      </c>
+      <c r="C29" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D29" s="12" t="inlineStr">
+        <is>
+          <t>T-041</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F29" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G29" s="16" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="12" t="inlineStr">
+        <is>
+          <t>I-30</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>Pending confirmations held in memory without expiry; lost on restart, break with &gt;1 instance (F2)</t>
+        </is>
+      </c>
+      <c r="C30" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D30" s="12" t="inlineStr">
+        <is>
+          <t>T-042</t>
+        </is>
+      </c>
+      <c r="E30" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F30" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G30" s="16" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="inlineStr">
+        <is>
+          <t>I-31</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>DESIGN still mentioned FastAPI / pytest after the switch to Java (F3)</t>
+        </is>
+      </c>
+      <c r="C31" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D31" s="12" t="inlineStr">
+        <is>
+          <t>Fixed in DESIGN 0.4.0</t>
+        </is>
+      </c>
+      <c r="E31" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F31" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G31" s="16" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>I-32</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>gh and ruff missing on the Mac</t>
+        </is>
+      </c>
+      <c r="C32" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D32" s="12" t="inlineStr">
+        <is>
+          <t>Installed 2026-10-03</t>
+        </is>
+      </c>
+      <c r="E32" s="12" t="inlineStr">
+        <is>
+          <t>Closed</t>
+        </is>
+      </c>
+      <c r="F32" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G32" s="16" t="n">
+        <v>46298</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>I-33</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>Agent blocked by the permission system from IAM grants and git pushes</t>
+        </is>
+      </c>
+      <c r="C33" s="12" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="D33" s="12" t="inlineStr">
+        <is>
+          <t>Owner runs the bootstrap apply and the branch push commands (session report)</t>
+        </is>
+      </c>
+      <c r="E33" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F33" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G33" s="16" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
+          <t>I-34</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>Artifact Registry 0.5 GB free tier for asia-south1 not verified</t>
+        </is>
+      </c>
+      <c r="C34" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D34" s="12" t="inlineStr">
+        <is>
+          <t>Check the pricing page before enabling app CD</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F34" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G34" s="16" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>I-35</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>gh not logged in; PR status and GitHub environments can't be managed</t>
+        </is>
+      </c>
+      <c r="C35" s="12" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D35" s="12" t="inlineStr">
+        <is>
+          <t>gh auth login</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="F35" s="16" t="n">
+        <v>46298</v>
+      </c>
+      <c r="G35" s="16" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:G7"/>

</xml_diff>